<commit_message>
Folders management and Empty regions exclusions
</commit_message>
<xml_diff>
--- a/GTAP12_matching.xlsx
+++ b/GTAP12_matching.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4cb83e15a8550b8f/Documenti/Claude projects/CC - Raccolta dati ENTICE/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4cb83e15a8550b8f/Documenti/GitHub/ENTICE_inventory/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="33" documentId="11_74A8CFD84E99951F1DBE718FA79E384DA9D36574" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A85A8A90-F69F-424E-B5F8-140FECB6C1C1}"/>
+  <xr:revisionPtr revIDLastSave="47" documentId="11_74A8CFD84E99951F1DBE718FA79E384DA9D36574" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AB2D0160-21C0-451E-B813-18B06E46F1D4}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Factor of production" sheetId="3" r:id="rId1"/>
@@ -861,15 +861,6 @@
     <t>International trade and transport margins</t>
   </si>
   <si>
-    <t>CAPITAL</t>
-  </si>
-  <si>
-    <t>LABOR</t>
-  </si>
-  <si>
-    <t>TAXES</t>
-  </si>
-  <si>
     <t>Lithium Cobalt Oxide batteries</t>
   </si>
   <si>
@@ -880,6 +871,15 @@
   </si>
   <si>
     <t>Manufacture of metallurgical silicon</t>
+  </si>
+  <si>
+    <t>Labor</t>
+  </si>
+  <si>
+    <t>Tax</t>
+  </si>
+  <si>
+    <t>TTM</t>
   </si>
 </sst>
 </file>
@@ -960,7 +960,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -973,7 +973,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1295,7 +1294,7 @@
         <v>261</v>
       </c>
       <c r="B2" t="s">
-        <v>275</v>
+        <v>262</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.35">
@@ -1303,7 +1302,7 @@
         <v>262</v>
       </c>
       <c r="B3" t="s">
-        <v>275</v>
+        <v>262</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.35">
@@ -1311,7 +1310,7 @@
         <v>263</v>
       </c>
       <c r="B4" t="s">
-        <v>275</v>
+        <v>262</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.35">
@@ -1319,7 +1318,7 @@
         <v>264</v>
       </c>
       <c r="B5" t="s">
-        <v>276</v>
+        <v>279</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.35">
@@ -1327,7 +1326,7 @@
         <v>265</v>
       </c>
       <c r="B6" t="s">
-        <v>276</v>
+        <v>279</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.35">
@@ -1335,7 +1334,7 @@
         <v>266</v>
       </c>
       <c r="B7" t="s">
-        <v>276</v>
+        <v>279</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.35">
@@ -1343,7 +1342,7 @@
         <v>267</v>
       </c>
       <c r="B8" t="s">
-        <v>276</v>
+        <v>279</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.35">
@@ -1351,7 +1350,7 @@
         <v>268</v>
       </c>
       <c r="B9" t="s">
-        <v>276</v>
+        <v>279</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.35">
@@ -1359,7 +1358,7 @@
         <v>269</v>
       </c>
       <c r="B10" t="s">
-        <v>277</v>
+        <v>280</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.35">
@@ -1367,7 +1366,7 @@
         <v>270</v>
       </c>
       <c r="B11" t="s">
-        <v>277</v>
+        <v>280</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.35">
@@ -1375,7 +1374,7 @@
         <v>271</v>
       </c>
       <c r="B12" t="s">
-        <v>277</v>
+        <v>280</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.35">
@@ -1383,7 +1382,7 @@
         <v>272</v>
       </c>
       <c r="B13" t="s">
-        <v>277</v>
+        <v>280</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.35">
@@ -1391,7 +1390,7 @@
         <v>273</v>
       </c>
       <c r="B14" t="s">
-        <v>277</v>
+        <v>280</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.35">
@@ -1399,7 +1398,7 @@
         <v>274</v>
       </c>
       <c r="B15" t="s">
-        <v>277</v>
+        <v>281</v>
       </c>
     </row>
   </sheetData>
@@ -2889,31 +2888,31 @@
     </row>
     <row r="185" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A185" t="s">
-        <v>278</v>
-      </c>
-      <c r="B185" s="6" t="s">
+        <v>275</v>
+      </c>
+      <c r="B185" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="186" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A186" t="s">
-        <v>279</v>
-      </c>
-      <c r="B186" s="6" t="s">
+        <v>276</v>
+      </c>
+      <c r="B186" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="187" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A187" t="s">
-        <v>280</v>
-      </c>
-      <c r="B187" s="6" t="s">
+        <v>277</v>
+      </c>
+      <c r="B187" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="188" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A188" t="s">
-        <v>281</v>
+        <v>278</v>
       </c>
       <c r="B188" t="s">
         <v>2</v>
@@ -2936,6 +2935,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x0101007BAED4C651AD5C4F9C61E3D439BD1465" ma:contentTypeVersion="11" ma:contentTypeDescription="Creare un nuovo documento." ma:contentTypeScope="" ma:versionID="3916dc5588df290b35e5c499b507bc33">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="90e7079a-7589-470d-892b-836f3f5ab9a4" xmlns:ns3="9ef6bf99-292f-445d-95df-6a8984d5eb85" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0e3fae628afbc47c424dc6703fd07071" ns2:_="" ns3:_="">
     <xsd:import namespace="90e7079a-7589-470d-892b-836f3f5ab9a4"/>
@@ -3130,15 +3138,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3AF17A8D-F061-4DE7-B3B8-B7DF39502DD5}">
   <ds:schemaRefs>
@@ -3151,6 +3150,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CCC7DBE7-124E-411E-99C5-C3E395F5B28C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F4B58489-93F8-4A04-91C4-4C320C5A26D1}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -3167,12 +3174,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CCC7DBE7-124E-411E-99C5-C3E395F5B28C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Relax unit-process checks; ignore Run.py
Update template checking logic and ignore Run.py in git.

- .gitignore: add Run.py to prevent committing local run/output script.
- template_checker.py:
  - Increase unit-process column-sum tolerance from 1e-4 to 1e-3 to reduce false positives.
  - Allow columns whose sum is ~0 to be kept if all retained values are zero; emit a warning when this exception is used.
  - Emit a warning when a unit-process row is missing a mapped input and is skipped.
  - Change total-production handling: Global rows are treated specially (skip in some checks) and zero-values are no longer universally skipped in region validation; also skip GLOBAL when comparing to GTAP.
-header fix in GTAP12_matching.xlsx
-automatic identification of the length of sectors column
</commit_message>
<xml_diff>
--- a/GTAP12_matching.xlsx
+++ b/GTAP12_matching.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4cb83e15a8550b8f/Documenti/GitHub/ENTICE_inventory/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="47" documentId="11_74A8CFD84E99951F1DBE718FA79E384DA9D36574" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AB2D0160-21C0-451E-B813-18B06E46F1D4}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{F229ADA7-0178-4BA1-B9EC-DC643AF4E5F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-60" yWindow="-16320" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Factor of production" sheetId="3" r:id="rId1"/>
@@ -816,9 +816,6 @@
     <t>GTAP12</t>
   </si>
   <si>
-    <t>GTAP EMTOCE</t>
-  </si>
-  <si>
     <t>Land</t>
   </si>
   <si>
@@ -880,6 +877,9 @@
   </si>
   <si>
     <t>TTM</t>
+  </si>
+  <si>
+    <t>GTAP ENTICE</t>
   </si>
 </sst>
 </file>
@@ -1291,114 +1291,114 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
+        <v>260</v>
+      </c>
+      <c r="B2" t="s">
         <v>261</v>
-      </c>
-      <c r="B2" t="s">
-        <v>262</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="B3" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="B4" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5" s="4" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="B5" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A6" s="4" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="B6" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A7" s="4" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="B7" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A8" s="4" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="B8" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A9" s="4" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="B9" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A10" s="4" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="B10" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A11" s="4" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="B11" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A12" s="4" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="B12" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A13" s="4" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="B13" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A14" s="4" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="B14" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A15" s="5" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="B15" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
     </row>
   </sheetData>
@@ -1416,7 +1416,7 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>260</v>
+        <v>281</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>259</v>
@@ -2888,7 +2888,7 @@
     </row>
     <row r="185" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A185" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="B185" t="s">
         <v>9</v>
@@ -2896,7 +2896,7 @@
     </row>
     <row r="186" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A186" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="B186" t="s">
         <v>9</v>
@@ -2904,7 +2904,7 @@
     </row>
     <row r="187" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A187" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="B187" t="s">
         <v>9</v>
@@ -2912,7 +2912,7 @@
     </row>
     <row r="188" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A188" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="B188" t="s">
         <v>2</v>
@@ -2935,15 +2935,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x0101007BAED4C651AD5C4F9C61E3D439BD1465" ma:contentTypeVersion="11" ma:contentTypeDescription="Creare un nuovo documento." ma:contentTypeScope="" ma:versionID="3916dc5588df290b35e5c499b507bc33">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="90e7079a-7589-470d-892b-836f3f5ab9a4" xmlns:ns3="9ef6bf99-292f-445d-95df-6a8984d5eb85" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0e3fae628afbc47c424dc6703fd07071" ns2:_="" ns3:_="">
     <xsd:import namespace="90e7079a-7589-470d-892b-836f3f5ab9a4"/>
@@ -3138,6 +3129,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3AF17A8D-F061-4DE7-B3B8-B7DF39502DD5}">
   <ds:schemaRefs>
@@ -3150,14 +3150,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CCC7DBE7-124E-411E-99C5-C3E395F5B28C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F4B58489-93F8-4A04-91C4-4C320C5A26D1}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -3174,4 +3166,12 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CCC7DBE7-124E-411E-99C5-C3E395F5B28C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Update GTAP matching workbook and inventory scripts
</commit_message>
<xml_diff>
--- a/GTAP12_matching.xlsx
+++ b/GTAP12_matching.xlsx
@@ -1,27 +1,30 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="11214"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4cb83e15a8550b8f/Documenti/GitHub/ENTICE_inventory/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lorenzorinaldi/Documents/GitHub/SESAM/ENTICE_inventory/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="11" documentId="11_D521553583E2E4D2E5CA9A41C5CB84CAA5A0B402" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DBB1D17F-7F49-4B08-870D-F24E2593347E}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{117F5E54-91C7-7147-8B6D-EB9BB88769B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="25600" windowHeight="19680" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Factor of production" sheetId="1" r:id="rId1"/>
     <sheet name="Sector" sheetId="2" r:id="rId2"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Sector!$A$1:$E$188</definedName>
+  </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="837" uniqueCount="443">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="837" uniqueCount="429">
   <si>
     <t>GTAP ENTICE</t>
   </si>
@@ -1085,6 +1088,9 @@
     <t>CNS</t>
   </si>
   <si>
+    <t>Trade</t>
+  </si>
+  <si>
     <t>TRD</t>
   </si>
   <si>
@@ -1305,51 +1311,6 @@
   </si>
   <si>
     <t>Manufacture of coke</t>
-  </si>
-  <si>
-    <t>land</t>
-  </si>
-  <si>
-    <t>capital</t>
-  </si>
-  <si>
-    <t>natlres</t>
-  </si>
-  <si>
-    <t>tech_aspros</t>
-  </si>
-  <si>
-    <t>clerks</t>
-  </si>
-  <si>
-    <t>service_shop</t>
-  </si>
-  <si>
-    <t>off_mgr_pros</t>
-  </si>
-  <si>
-    <t>ag_othlowsk</t>
-  </si>
-  <si>
-    <t>ptax</t>
-  </si>
-  <si>
-    <t>idtax</t>
-  </si>
-  <si>
-    <t>imtax</t>
-  </si>
-  <si>
-    <t>etax</t>
-  </si>
-  <si>
-    <t>mtax</t>
-  </si>
-  <si>
-    <t>ittm</t>
-  </si>
-  <si>
-    <t>Wholesale and retail trade, repair</t>
   </si>
 </sst>
 </file>
@@ -1760,14 +1721,14 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:C29"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:C15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="57.1796875" style="5" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="57.1640625" style="5" bestFit="1" customWidth="1"/>
     <col min="2" max="3" width="13" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B1" s="2" t="s">
         <v>2</v>
       </c>
@@ -1775,270 +1736,158 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="5" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="B2" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="C2" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="5" t="s">
         <v>404</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="5" t="s">
-        <v>403</v>
-      </c>
       <c r="B3" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="C3" t="s">
-        <v>405</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+        <v>406</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="5" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="B4" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="C4" t="s">
-        <v>407</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+        <v>408</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="6" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="B5" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="C5" t="s">
+        <v>411</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="6" t="s">
+        <v>412</v>
+      </c>
+      <c r="B6" t="s">
         <v>410</v>
       </c>
-    </row>
-    <row r="6" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="6" t="s">
+      <c r="C6" t="s">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="6" t="s">
+        <v>414</v>
+      </c>
+      <c r="B7" t="s">
+        <v>410</v>
+      </c>
+      <c r="C7" t="s">
+        <v>415</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="6" t="s">
+        <v>416</v>
+      </c>
+      <c r="B8" t="s">
+        <v>410</v>
+      </c>
+      <c r="C8" t="s">
         <v>411</v>
       </c>
-      <c r="B6" t="s">
-        <v>409</v>
-      </c>
-      <c r="C6" t="s">
-        <v>412</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="6" t="s">
-        <v>413</v>
-      </c>
-      <c r="B7" t="s">
-        <v>409</v>
-      </c>
-      <c r="C7" t="s">
-        <v>414</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="6" t="s">
+    </row>
+    <row r="9" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A9" s="6" t="s">
+        <v>417</v>
+      </c>
+      <c r="B9" t="s">
+        <v>410</v>
+      </c>
+      <c r="C9" t="s">
         <v>415</v>
       </c>
-      <c r="B8" t="s">
-        <v>409</v>
-      </c>
-      <c r="C8" t="s">
-        <v>410</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="6" t="s">
-        <v>416</v>
-      </c>
-      <c r="B9" t="s">
-        <v>409</v>
-      </c>
-      <c r="C9" t="s">
-        <v>414</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    </row>
+    <row r="10" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="6" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="B10" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="C10" t="s">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A11" s="6" t="s">
+        <v>421</v>
+      </c>
+      <c r="B11" t="s">
         <v>419</v>
       </c>
-    </row>
-    <row r="11" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="6" t="s">
-        <v>420</v>
-      </c>
-      <c r="B11" t="s">
-        <v>418</v>
-      </c>
       <c r="C11" t="s">
-        <v>421</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="6" t="s">
+        <v>423</v>
+      </c>
+      <c r="B12" t="s">
+        <v>419</v>
+      </c>
+      <c r="C12" t="s">
         <v>422</v>
       </c>
-      <c r="B12" t="s">
-        <v>418</v>
-      </c>
-      <c r="C12" t="s">
-        <v>421</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    </row>
+    <row r="13" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="6" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="B13" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="C13" t="s">
-        <v>421</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="6" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="B14" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="C14" t="s">
-        <v>421</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="4" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="B15" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="C15" t="s">
-        <v>421</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A16" s="5" t="s">
-        <v>428</v>
-      </c>
-      <c r="B16" t="s">
-        <v>403</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A17" s="5" t="s">
-        <v>429</v>
-      </c>
-      <c r="B17" t="s">
-        <v>403</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A18" s="5" t="s">
-        <v>430</v>
-      </c>
-      <c r="B18" t="s">
-        <v>403</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A19" s="5" t="s">
-        <v>431</v>
-      </c>
-      <c r="B19" t="s">
-        <v>409</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A20" s="5" t="s">
-        <v>432</v>
-      </c>
-      <c r="B20" t="s">
-        <v>409</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A21" s="5" t="s">
-        <v>433</v>
-      </c>
-      <c r="B21" t="s">
-        <v>409</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A22" s="5" t="s">
-        <v>434</v>
-      </c>
-      <c r="B22" t="s">
-        <v>409</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A23" s="5" t="s">
-        <v>435</v>
-      </c>
-      <c r="B23" t="s">
-        <v>409</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A24" s="5" t="s">
-        <v>436</v>
-      </c>
-      <c r="B24" t="s">
-        <v>418</v>
-      </c>
-    </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A25" s="5" t="s">
-        <v>437</v>
-      </c>
-      <c r="B25" t="s">
-        <v>418</v>
-      </c>
-    </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A26" s="5" t="s">
-        <v>438</v>
-      </c>
-      <c r="B26" t="s">
-        <v>418</v>
-      </c>
-    </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A27" s="5" t="s">
-        <v>439</v>
-      </c>
-      <c r="B27" t="s">
-        <v>418</v>
-      </c>
-    </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A28" s="5" t="s">
-        <v>440</v>
-      </c>
-      <c r="B28" t="s">
-        <v>418</v>
-      </c>
-    </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A29" s="5" t="s">
-        <v>441</v>
-      </c>
-      <c r="B29" t="s">
-        <v>426</v>
+        <v>422</v>
       </c>
     </row>
   </sheetData>
@@ -2052,16 +1901,16 @@
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:E189"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="102.26953125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.7265625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="102.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.6640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="13" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.26953125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.83203125" customWidth="1"/>
     <col min="5" max="5" width="13" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2078,7 +1927,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -2092,7 +1941,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>7</v>
       </c>
@@ -2106,7 +1955,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -2120,7 +1969,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -2134,7 +1983,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>11</v>
       </c>
@@ -2148,7 +1997,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>14</v>
       </c>
@@ -2162,7 +2011,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>16</v>
       </c>
@@ -2176,7 +2025,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>18</v>
       </c>
@@ -2190,7 +2039,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="10" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>20</v>
       </c>
@@ -2204,7 +2053,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="11" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>22</v>
       </c>
@@ -2218,7 +2067,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="12" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>25</v>
       </c>
@@ -2232,7 +2081,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="13" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>27</v>
       </c>
@@ -2246,7 +2095,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="14" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>29</v>
       </c>
@@ -2260,7 +2109,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="15" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>31</v>
       </c>
@@ -2274,7 +2123,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="16" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>33</v>
       </c>
@@ -2288,7 +2137,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="17" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>36</v>
       </c>
@@ -2302,7 +2151,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="18" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>38</v>
       </c>
@@ -2316,7 +2165,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="19" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>40</v>
       </c>
@@ -2330,7 +2179,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="20" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>42</v>
       </c>
@@ -2344,7 +2193,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="21" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>44</v>
       </c>
@@ -2358,7 +2207,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="22" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>46</v>
       </c>
@@ -2372,7 +2221,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="23" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>48</v>
       </c>
@@ -2386,7 +2235,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="24" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>50</v>
       </c>
@@ -2400,7 +2249,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="25" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>52</v>
       </c>
@@ -2414,7 +2263,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="26" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>54</v>
       </c>
@@ -2428,7 +2277,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="27" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>56</v>
       </c>
@@ -2442,7 +2291,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="28" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>58</v>
       </c>
@@ -2456,7 +2305,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="29" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>61</v>
       </c>
@@ -2470,7 +2319,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="30" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>63</v>
       </c>
@@ -2484,7 +2333,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="31" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>65</v>
       </c>
@@ -2498,7 +2347,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="32" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>67</v>
       </c>
@@ -2512,7 +2361,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="33" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>69</v>
       </c>
@@ -2526,7 +2375,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="34" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>71</v>
       </c>
@@ -2540,7 +2389,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="35" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>73</v>
       </c>
@@ -2554,7 +2403,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="36" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>76</v>
       </c>
@@ -2568,7 +2417,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="37" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>78</v>
       </c>
@@ -2582,7 +2431,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="38" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>80</v>
       </c>
@@ -2596,7 +2445,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="39" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>82</v>
       </c>
@@ -2610,7 +2459,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="40" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>84</v>
       </c>
@@ -2624,7 +2473,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="41" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>86</v>
       </c>
@@ -2638,7 +2487,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="42" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>88</v>
       </c>
@@ -2652,7 +2501,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="43" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>90</v>
       </c>
@@ -2666,7 +2515,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="44" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>92</v>
       </c>
@@ -2680,7 +2529,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="45" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>94</v>
       </c>
@@ -2694,7 +2543,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="46" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
         <v>96</v>
       </c>
@@ -2708,7 +2557,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="47" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
         <v>98</v>
       </c>
@@ -2722,7 +2571,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="48" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
         <v>102</v>
       </c>
@@ -2735,8 +2584,11 @@
       <c r="D48" t="s">
         <v>104</v>
       </c>
-    </row>
-    <row r="49" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E48" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
         <v>105</v>
       </c>
@@ -2749,8 +2601,11 @@
       <c r="D49" t="s">
         <v>104</v>
       </c>
-    </row>
-    <row r="50" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E49" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
         <v>107</v>
       </c>
@@ -2767,7 +2622,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="51" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
         <v>110</v>
       </c>
@@ -2780,8 +2635,11 @@
       <c r="D51" t="s">
         <v>104</v>
       </c>
-    </row>
-    <row r="52" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E51" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
         <v>112</v>
       </c>
@@ -2794,8 +2652,11 @@
       <c r="D52" t="s">
         <v>114</v>
       </c>
-    </row>
-    <row r="53" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E52" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
         <v>115</v>
       </c>
@@ -2808,8 +2669,11 @@
       <c r="D53" t="s">
         <v>104</v>
       </c>
-    </row>
-    <row r="54" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E53" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
         <v>117</v>
       </c>
@@ -2822,8 +2686,11 @@
       <c r="D54" t="s">
         <v>104</v>
       </c>
-    </row>
-    <row r="55" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E54" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
         <v>119</v>
       </c>
@@ -2836,8 +2703,11 @@
       <c r="D55" t="s">
         <v>104</v>
       </c>
-    </row>
-    <row r="56" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E55" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
         <v>121</v>
       </c>
@@ -2850,8 +2720,11 @@
       <c r="D56" t="s">
         <v>104</v>
       </c>
-    </row>
-    <row r="57" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E56" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
         <v>123</v>
       </c>
@@ -2864,8 +2737,11 @@
       <c r="D57" t="s">
         <v>125</v>
       </c>
-    </row>
-    <row r="58" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E57" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="58" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
         <v>126</v>
       </c>
@@ -2882,7 +2758,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="59" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
         <v>128</v>
       </c>
@@ -2899,7 +2775,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="60" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
         <v>130</v>
       </c>
@@ -2916,7 +2792,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="61" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
         <v>132</v>
       </c>
@@ -2933,7 +2809,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="62" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
         <v>134</v>
       </c>
@@ -2947,7 +2823,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="63" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
         <v>136</v>
       </c>
@@ -2960,8 +2836,11 @@
       <c r="D63" t="s">
         <v>101</v>
       </c>
-    </row>
-    <row r="64" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E63" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
         <v>138</v>
       </c>
@@ -2974,8 +2853,11 @@
       <c r="D64" t="s">
         <v>104</v>
       </c>
-    </row>
-    <row r="65" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E64" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="65" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
         <v>140</v>
       </c>
@@ -2989,7 +2871,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="66" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
         <v>141</v>
       </c>
@@ -3003,7 +2885,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="67" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
         <v>143</v>
       </c>
@@ -3016,8 +2898,11 @@
       <c r="D67" t="s">
         <v>101</v>
       </c>
-    </row>
-    <row r="68" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E67" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="68" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
         <v>145</v>
       </c>
@@ -3031,7 +2916,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="69" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
         <v>147</v>
       </c>
@@ -3045,7 +2930,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="70" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
         <v>148</v>
       </c>
@@ -3059,7 +2944,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="71" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
         <v>150</v>
       </c>
@@ -3073,7 +2958,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="72" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
         <v>152</v>
       </c>
@@ -3087,7 +2972,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="73" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
         <v>154</v>
       </c>
@@ -3101,7 +2986,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="74" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
         <v>156</v>
       </c>
@@ -3115,7 +3000,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="75" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A75" t="s">
         <v>158</v>
       </c>
@@ -3129,7 +3014,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="76" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
         <v>160</v>
       </c>
@@ -3143,7 +3028,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="77" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
         <v>162</v>
       </c>
@@ -3157,7 +3042,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="78" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A78" t="s">
         <v>164</v>
       </c>
@@ -3171,7 +3056,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="79" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A79" t="s">
         <v>166</v>
       </c>
@@ -3185,7 +3070,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="80" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A80" t="s">
         <v>168</v>
       </c>
@@ -3199,7 +3084,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="81" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A81" t="s">
         <v>170</v>
       </c>
@@ -3210,10 +3095,10 @@
         <v>172</v>
       </c>
       <c r="D81" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="82" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="82" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A82" t="s">
         <v>174</v>
       </c>
@@ -3224,10 +3109,10 @@
         <v>172</v>
       </c>
       <c r="D82" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="83" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="83" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A83" t="s">
         <v>175</v>
       </c>
@@ -3241,7 +3126,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="84" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A84" t="s">
         <v>179</v>
       </c>
@@ -3255,7 +3140,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="85" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A85" t="s">
         <v>181</v>
       </c>
@@ -3269,7 +3154,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="86" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A86" t="s">
         <v>183</v>
       </c>
@@ -3283,7 +3168,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="87" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A87" t="s">
         <v>185</v>
       </c>
@@ -3297,7 +3182,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="88" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A88" t="s">
         <v>187</v>
       </c>
@@ -3311,7 +3196,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="89" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A89" t="s">
         <v>189</v>
       </c>
@@ -3324,8 +3209,11 @@
       <c r="D89" t="s">
         <v>178</v>
       </c>
-    </row>
-    <row r="90" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E89" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="90" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A90" t="s">
         <v>191</v>
       </c>
@@ -3338,8 +3226,11 @@
       <c r="D90" t="s">
         <v>178</v>
       </c>
-    </row>
-    <row r="91" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E90" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="91" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A91" t="s">
         <v>193</v>
       </c>
@@ -3352,8 +3243,11 @@
       <c r="D91" t="s">
         <v>178</v>
       </c>
-    </row>
-    <row r="92" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E91" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="92" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A92" t="s">
         <v>195</v>
       </c>
@@ -3366,8 +3260,11 @@
       <c r="D92" t="s">
         <v>178</v>
       </c>
-    </row>
-    <row r="93" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E92" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="93" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A93" t="s">
         <v>197</v>
       </c>
@@ -3380,8 +3277,11 @@
       <c r="D93" t="s">
         <v>178</v>
       </c>
-    </row>
-    <row r="94" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E93" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="94" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A94" t="s">
         <v>199</v>
       </c>
@@ -3394,8 +3294,11 @@
       <c r="D94" t="s">
         <v>178</v>
       </c>
-    </row>
-    <row r="95" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E94" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="95" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A95" t="s">
         <v>201</v>
       </c>
@@ -3408,8 +3311,11 @@
       <c r="D95" t="s">
         <v>203</v>
       </c>
-    </row>
-    <row r="96" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E95" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="96" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A96" t="s">
         <v>204</v>
       </c>
@@ -3422,8 +3328,11 @@
       <c r="D96" t="s">
         <v>178</v>
       </c>
-    </row>
-    <row r="97" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E96" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="97" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A97" t="s">
         <v>206</v>
       </c>
@@ -3436,8 +3345,11 @@
       <c r="D97" t="s">
         <v>178</v>
       </c>
-    </row>
-    <row r="98" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E97" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="98" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A98" t="s">
         <v>208</v>
       </c>
@@ -3450,8 +3362,11 @@
       <c r="D98" t="s">
         <v>178</v>
       </c>
-    </row>
-    <row r="99" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E98" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="99" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A99" t="s">
         <v>210</v>
       </c>
@@ -3465,7 +3380,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="100" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A100" t="s">
         <v>212</v>
       </c>
@@ -3482,7 +3397,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="101" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A101" t="s">
         <v>214</v>
       </c>
@@ -3495,8 +3410,11 @@
       <c r="D101" t="s">
         <v>216</v>
       </c>
-    </row>
-    <row r="102" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E101" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="102" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A102" t="s">
         <v>217</v>
       </c>
@@ -3509,8 +3427,11 @@
       <c r="D102" t="s">
         <v>216</v>
       </c>
-    </row>
-    <row r="103" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E102" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="103" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A103" t="s">
         <v>219</v>
       </c>
@@ -3524,7 +3445,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="104" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A104" t="s">
         <v>221</v>
       </c>
@@ -3538,7 +3459,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="105" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A105" t="s">
         <v>224</v>
       </c>
@@ -3552,7 +3473,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="106" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A106" t="s">
         <v>226</v>
       </c>
@@ -3566,7 +3487,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="107" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A107" t="s">
         <v>228</v>
       </c>
@@ -3580,7 +3501,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="108" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A108" t="s">
         <v>231</v>
       </c>
@@ -3594,7 +3515,7 @@
         <v>234</v>
       </c>
     </row>
-    <row r="109" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A109" t="s">
         <v>235</v>
       </c>
@@ -3608,7 +3529,7 @@
         <v>234</v>
       </c>
     </row>
-    <row r="110" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A110" t="s">
         <v>237</v>
       </c>
@@ -3622,7 +3543,7 @@
         <v>233</v>
       </c>
     </row>
-    <row r="111" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A111" t="s">
         <v>239</v>
       </c>
@@ -3636,7 +3557,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="112" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A112" t="s">
         <v>243</v>
       </c>
@@ -3650,7 +3571,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="113" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A113" t="s">
         <v>245</v>
       </c>
@@ -3664,7 +3585,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="114" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A114" t="s">
         <v>247</v>
       </c>
@@ -3678,7 +3599,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="115" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A115" t="s">
         <v>249</v>
       </c>
@@ -3692,7 +3613,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="116" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A116" t="s">
         <v>251</v>
       </c>
@@ -3706,7 +3627,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="117" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A117" t="s">
         <v>252</v>
       </c>
@@ -3720,7 +3641,7 @@
         <v>253</v>
       </c>
     </row>
-    <row r="118" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A118" t="s">
         <v>254</v>
       </c>
@@ -3734,7 +3655,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="119" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A119" t="s">
         <v>256</v>
       </c>
@@ -3748,7 +3669,7 @@
         <v>259</v>
       </c>
     </row>
-    <row r="120" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A120" t="s">
         <v>260</v>
       </c>
@@ -3762,7 +3683,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="121" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A121" t="s">
         <v>262</v>
       </c>
@@ -3776,7 +3697,7 @@
         <v>263</v>
       </c>
     </row>
-    <row r="122" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A122" t="s">
         <v>264</v>
       </c>
@@ -3790,7 +3711,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="123" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A123" t="s">
         <v>266</v>
       </c>
@@ -3807,7 +3728,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="124" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A124" t="s">
         <v>268</v>
       </c>
@@ -3824,7 +3745,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="125" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A125" t="s">
         <v>270</v>
       </c>
@@ -3837,8 +3758,11 @@
       <c r="D125" t="s">
         <v>230</v>
       </c>
-    </row>
-    <row r="126" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E125" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="126" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A126" t="s">
         <v>272</v>
       </c>
@@ -3851,8 +3775,11 @@
       <c r="D126" t="s">
         <v>274</v>
       </c>
-    </row>
-    <row r="127" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E126" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="127" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A127" t="s">
         <v>275</v>
       </c>
@@ -3865,8 +3792,11 @@
       <c r="D127" t="s">
         <v>277</v>
       </c>
-    </row>
-    <row r="128" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E127" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="128" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A128" t="s">
         <v>278</v>
       </c>
@@ -3879,8 +3809,11 @@
       <c r="D128" t="s">
         <v>277</v>
       </c>
-    </row>
-    <row r="129" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E128" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="129" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A129" t="s">
         <v>280</v>
       </c>
@@ -3894,7 +3827,7 @@
         <v>274</v>
       </c>
     </row>
-    <row r="130" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A130" t="s">
         <v>282</v>
       </c>
@@ -3908,7 +3841,7 @@
         <v>283</v>
       </c>
     </row>
-    <row r="131" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A131" t="s">
         <v>284</v>
       </c>
@@ -3922,7 +3855,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="132" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A132" t="s">
         <v>287</v>
       </c>
@@ -3936,7 +3869,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="133" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A133" t="s">
         <v>289</v>
       </c>
@@ -3950,7 +3883,7 @@
         <v>291</v>
       </c>
     </row>
-    <row r="134" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A134" t="s">
         <v>292</v>
       </c>
@@ -3964,7 +3897,7 @@
         <v>291</v>
       </c>
     </row>
-    <row r="135" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A135" t="s">
         <v>294</v>
       </c>
@@ -3978,7 +3911,7 @@
         <v>291</v>
       </c>
     </row>
-    <row r="136" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A136" t="s">
         <v>296</v>
       </c>
@@ -3992,7 +3925,7 @@
         <v>291</v>
       </c>
     </row>
-    <row r="137" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A137" t="s">
         <v>298</v>
       </c>
@@ -4006,7 +3939,7 @@
         <v>291</v>
       </c>
     </row>
-    <row r="138" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A138" t="s">
         <v>300</v>
       </c>
@@ -4020,7 +3953,7 @@
         <v>291</v>
       </c>
     </row>
-    <row r="139" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A139" t="s">
         <v>302</v>
       </c>
@@ -4034,7 +3967,7 @@
         <v>299</v>
       </c>
     </row>
-    <row r="140" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A140" t="s">
         <v>304</v>
       </c>
@@ -4048,7 +3981,7 @@
         <v>306</v>
       </c>
     </row>
-    <row r="141" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A141" t="s">
         <v>307</v>
       </c>
@@ -4062,7 +3995,7 @@
         <v>306</v>
       </c>
     </row>
-    <row r="142" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="142" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A142" t="s">
         <v>309</v>
       </c>
@@ -4076,7 +4009,7 @@
         <v>306</v>
       </c>
     </row>
-    <row r="143" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="143" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A143" t="s">
         <v>311</v>
       </c>
@@ -4090,7 +4023,7 @@
         <v>306</v>
       </c>
     </row>
-    <row r="144" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A144" t="s">
         <v>313</v>
       </c>
@@ -4104,7 +4037,7 @@
         <v>306</v>
       </c>
     </row>
-    <row r="145" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A145" t="s">
         <v>315</v>
       </c>
@@ -4118,7 +4051,7 @@
         <v>306</v>
       </c>
     </row>
-    <row r="146" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A146" t="s">
         <v>317</v>
       </c>
@@ -4132,7 +4065,7 @@
         <v>306</v>
       </c>
     </row>
-    <row r="147" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A147" t="s">
         <v>319</v>
       </c>
@@ -4146,7 +4079,7 @@
         <v>320</v>
       </c>
     </row>
-    <row r="148" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A148" t="s">
         <v>321</v>
       </c>
@@ -4160,7 +4093,7 @@
         <v>322</v>
       </c>
     </row>
-    <row r="149" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A149" t="s">
         <v>323</v>
       </c>
@@ -4174,7 +4107,7 @@
         <v>325</v>
       </c>
     </row>
-    <row r="150" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="150" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A150" t="s">
         <v>326</v>
       </c>
@@ -4188,7 +4121,7 @@
         <v>325</v>
       </c>
     </row>
-    <row r="151" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A151" t="s">
         <v>328</v>
       </c>
@@ -4202,7 +4135,7 @@
         <v>325</v>
       </c>
     </row>
-    <row r="152" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="152" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A152" t="s">
         <v>330</v>
       </c>
@@ -4216,7 +4149,7 @@
         <v>325</v>
       </c>
     </row>
-    <row r="153" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="153" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A153" t="s">
         <v>332</v>
       </c>
@@ -4230,7 +4163,7 @@
         <v>325</v>
       </c>
     </row>
-    <row r="154" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="154" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A154" t="s">
         <v>334</v>
       </c>
@@ -4244,7 +4177,7 @@
         <v>325</v>
       </c>
     </row>
-    <row r="155" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="155" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A155" t="s">
         <v>336</v>
       </c>
@@ -4258,7 +4191,7 @@
         <v>325</v>
       </c>
     </row>
-    <row r="156" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="156" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A156" t="s">
         <v>338</v>
       </c>
@@ -4272,7 +4205,7 @@
         <v>325</v>
       </c>
     </row>
-    <row r="157" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="157" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A157" t="s">
         <v>340</v>
       </c>
@@ -4286,7 +4219,7 @@
         <v>325</v>
       </c>
     </row>
-    <row r="158" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="158" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A158" t="s">
         <v>342</v>
       </c>
@@ -4300,7 +4233,7 @@
         <v>325</v>
       </c>
     </row>
-    <row r="159" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="159" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A159" t="s">
         <v>344</v>
       </c>
@@ -4314,7 +4247,7 @@
         <v>325</v>
       </c>
     </row>
-    <row r="160" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="160" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A160" t="s">
         <v>346</v>
       </c>
@@ -4328,7 +4261,7 @@
         <v>325</v>
       </c>
     </row>
-    <row r="161" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="161" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A161" t="s">
         <v>348</v>
       </c>
@@ -4342,7 +4275,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="162" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="162" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A162" t="s">
         <v>350</v>
       </c>
@@ -4356,7 +4289,7 @@
         <v>351</v>
       </c>
     </row>
-    <row r="163" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="163" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A163" t="s">
         <v>352</v>
       </c>
@@ -4370,307 +4303,307 @@
         <v>353</v>
       </c>
     </row>
-    <row r="164" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A164" t="s">
-        <v>442</v>
+    <row r="164" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A164" s="3" t="s">
+        <v>354</v>
       </c>
       <c r="B164" s="3" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="C164" s="3" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="D164" t="s">
-        <v>354</v>
-      </c>
-    </row>
-    <row r="165" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="165" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A165" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="B165" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="C165" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="D165" t="s">
-        <v>356</v>
-      </c>
-    </row>
-    <row r="166" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="166" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A166" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="B166" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="C166" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="D166" t="s">
-        <v>359</v>
-      </c>
-    </row>
-    <row r="167" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="167" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A167" t="s">
+        <v>361</v>
+      </c>
+      <c r="B167" t="s">
+        <v>362</v>
+      </c>
+      <c r="C167" t="s">
         <v>360</v>
       </c>
-      <c r="B167" t="s">
-        <v>361</v>
-      </c>
-      <c r="C167" t="s">
-        <v>359</v>
-      </c>
       <c r="D167" t="s">
-        <v>359</v>
-      </c>
-    </row>
-    <row r="168" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="168" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A168" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="B168" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="C168" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="D168" t="s">
-        <v>359</v>
-      </c>
-    </row>
-    <row r="169" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="169" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A169" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="B169" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="C169" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="D169" t="s">
-        <v>359</v>
-      </c>
-    </row>
-    <row r="170" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="170" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A170" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="B170" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="C170" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="D170" t="s">
-        <v>367</v>
-      </c>
-    </row>
-    <row r="171" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+        <v>368</v>
+      </c>
+    </row>
+    <row r="171" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A171" t="s">
+        <v>369</v>
+      </c>
+      <c r="B171" t="s">
         <v>368</v>
       </c>
-      <c r="B171" t="s">
-        <v>367</v>
-      </c>
       <c r="C171" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="D171" t="s">
-        <v>367</v>
-      </c>
-    </row>
-    <row r="172" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+        <v>368</v>
+      </c>
+    </row>
+    <row r="172" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A172" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="B172" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="C172" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="D172" t="s">
-        <v>367</v>
-      </c>
-    </row>
-    <row r="173" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+        <v>368</v>
+      </c>
+    </row>
+    <row r="173" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A173" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="B173" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="C173" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="D173" t="s">
-        <v>371</v>
-      </c>
-    </row>
-    <row r="174" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="174" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A174" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="B174" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="C174" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="D174" t="s">
-        <v>373</v>
-      </c>
-    </row>
-    <row r="175" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="175" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A175" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="B175" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="C175" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="D175" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="176" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="176" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A176" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="B176" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="C176" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="D176" t="s">
-        <v>377</v>
-      </c>
-    </row>
-    <row r="177" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+        <v>378</v>
+      </c>
+    </row>
+    <row r="177" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A177" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="B177" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="C177" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="D177" t="s">
-        <v>379</v>
-      </c>
-    </row>
-    <row r="178" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="178" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A178" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="B178" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="C178" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="D178" t="s">
-        <v>381</v>
-      </c>
-    </row>
-    <row r="179" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+        <v>382</v>
+      </c>
+    </row>
+    <row r="179" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A179" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="B179" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="C179" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="D179" t="s">
-        <v>383</v>
-      </c>
-    </row>
-    <row r="180" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+        <v>384</v>
+      </c>
+    </row>
+    <row r="180" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A180" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="B180" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="C180" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="D180" t="s">
-        <v>385</v>
-      </c>
-    </row>
-    <row r="181" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="181" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A181" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="B181" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="C181" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="D181" t="s">
-        <v>387</v>
-      </c>
-    </row>
-    <row r="182" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+        <v>388</v>
+      </c>
+    </row>
+    <row r="182" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A182" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="B182" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="C182" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="D182" t="s">
-        <v>389</v>
-      </c>
-    </row>
-    <row r="183" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="183" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A183" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="B183" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="C183" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="D183" t="s">
-        <v>391</v>
-      </c>
-    </row>
-    <row r="184" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+        <v>392</v>
+      </c>
+    </row>
+    <row r="184" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A184" s="4" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="B184" s="4" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="C184" s="4" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="D184" s="4" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="E184" s="4"/>
     </row>
-    <row r="185" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="185" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A185" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="B185" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="C185" t="s">
         <v>291</v>
@@ -4679,12 +4612,12 @@
         <v>291</v>
       </c>
     </row>
-    <row r="186" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="186" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A186" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="B186" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="C186" t="s">
         <v>291</v>
@@ -4693,12 +4626,12 @@
         <v>291</v>
       </c>
     </row>
-    <row r="187" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="187" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A187" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="B187" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="C187" t="s">
         <v>291</v>
@@ -4707,12 +4640,12 @@
         <v>291</v>
       </c>
     </row>
-    <row r="188" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="188" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A188" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="B188" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="C188" t="s">
         <v>177</v>
@@ -4721,9 +4654,9 @@
         <v>178</v>
       </c>
     </row>
-    <row r="189" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="189" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A189" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="B189" t="s">
         <v>173</v>
@@ -4736,6 +4669,7 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:E188" xr:uid="{00000000-0001-0000-0100-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
latest devs up to final exporter in d2.4 format
</commit_message>
<xml_diff>
--- a/GTAP12_matching.xlsx
+++ b/GTAP12_matching.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lorenzorinaldi/Documents/GitHub/SESAM/ENTICE_inventory/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{117F5E54-91C7-7147-8B6D-EB9BB88769B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65DF75F7-F797-F740-BAE0-03864FDF7C3C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="25600" windowHeight="19680" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,14 +17,14 @@
     <sheet name="Sector" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Sector!$A$1:$E$188</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Sector!$A$1:$E$190</definedName>
   </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="837" uniqueCount="429">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="846" uniqueCount="431">
   <si>
     <t>GTAP ENTICE</t>
   </si>
@@ -449,868 +449,874 @@
     <t>Mining of silicon</t>
   </si>
   <si>
+    <t>CPH</t>
+  </si>
+  <si>
+    <t>Mining of natural magnesium carbonate "magnesite"+magnesia, fused or dead-burned (sintered)</t>
+  </si>
+  <si>
+    <t>MGC</t>
+  </si>
+  <si>
+    <t>Manufacture of bovine meat products</t>
+  </si>
+  <si>
+    <t>CMT</t>
+  </si>
+  <si>
+    <t>Manufacture of meat products nec</t>
+  </si>
+  <si>
+    <t>Manufacture of vegetable oils and fats</t>
+  </si>
+  <si>
+    <t>VOL</t>
+  </si>
+  <si>
+    <t>Manufacture of dairy products</t>
+  </si>
+  <si>
+    <t>MIL</t>
+  </si>
+  <si>
+    <t>Manufacture of processed rice</t>
+  </si>
+  <si>
+    <t>PCR</t>
+  </si>
+  <si>
+    <t>Manufacture of sugar</t>
+  </si>
+  <si>
+    <t>SGR</t>
+  </si>
+  <si>
+    <t>Manufacture of food products nec</t>
+  </si>
+  <si>
+    <t>OFD</t>
+  </si>
+  <si>
+    <t>Manufacture of beverages and tobacco products</t>
+  </si>
+  <si>
+    <t>B_T</t>
+  </si>
+  <si>
+    <t>Manufacture of textiles</t>
+  </si>
+  <si>
+    <t>TEX</t>
+  </si>
+  <si>
+    <t>Manufacture of wearing apparel</t>
+  </si>
+  <si>
+    <t>WAP</t>
+  </si>
+  <si>
+    <t>Manufacture of leather products</t>
+  </si>
+  <si>
+    <t>LEA</t>
+  </si>
+  <si>
+    <t>Manufacture of wood products</t>
+  </si>
+  <si>
+    <t>LUM</t>
+  </si>
+  <si>
+    <t>Manufacture of paper products, publishing</t>
+  </si>
+  <si>
+    <t>PPP</t>
+  </si>
+  <si>
+    <t>Manufacture of petroleum products</t>
+  </si>
+  <si>
+    <t>PEP</t>
+  </si>
+  <si>
+    <t>P_C</t>
+  </si>
+  <si>
+    <t>PCP</t>
+  </si>
+  <si>
+    <t>Manufacture of coal products</t>
+  </si>
+  <si>
+    <t>Manufacture of other chemicals</t>
+  </si>
+  <si>
+    <t>XCH</t>
+  </si>
+  <si>
+    <t>CHM</t>
+  </si>
+  <si>
+    <t>XCH_BPH</t>
+  </si>
+  <si>
+    <t>Manufacture of ammonia</t>
+  </si>
+  <si>
+    <t>AMM</t>
+  </si>
+  <si>
+    <t>Manufacture of hydrogen via electrolysis</t>
+  </si>
+  <si>
+    <t>HYE</t>
+  </si>
+  <si>
+    <t>Manufacture of hydrogen via steam reforming</t>
+  </si>
+  <si>
+    <t>HYS</t>
+  </si>
+  <si>
+    <t>Manufacture of methanol</t>
+  </si>
+  <si>
+    <t>MTH</t>
+  </si>
+  <si>
+    <t>Manufacture of high value chemicals</t>
+  </si>
+  <si>
+    <t>HVC</t>
+  </si>
+  <si>
+    <t>Manufacture of artificial graphite</t>
+  </si>
+  <si>
+    <t>AGT</t>
+  </si>
+  <si>
+    <t>Manufacture of refined lithium</t>
+  </si>
+  <si>
+    <t>LIR</t>
+  </si>
+  <si>
+    <t>Manufacture of refined rare earths</t>
+  </si>
+  <si>
+    <t>RER</t>
+  </si>
+  <si>
+    <t>Manufacture of refined manganese</t>
+  </si>
+  <si>
+    <t>MNR</t>
+  </si>
+  <si>
+    <t>Manufacture of refined nickel</t>
+  </si>
+  <si>
+    <t>NIR</t>
+  </si>
+  <si>
+    <t>Manufacture of refined cobalt</t>
+  </si>
+  <si>
+    <t>COR</t>
+  </si>
+  <si>
+    <t>Manufacture of refined zinc</t>
+  </si>
+  <si>
+    <t>ZIR</t>
+  </si>
+  <si>
+    <t>LZR</t>
+  </si>
+  <si>
+    <t>Manufacture of refined chromium</t>
+  </si>
+  <si>
+    <t>CRR</t>
+  </si>
+  <si>
+    <t>Manufacture of refined titanium</t>
+  </si>
+  <si>
+    <t>TIR</t>
+  </si>
+  <si>
+    <t>Manufacture of refined gallium</t>
+  </si>
+  <si>
+    <t>GAR</t>
+  </si>
+  <si>
+    <t>Manufacture of refined magnesium</t>
+  </si>
+  <si>
+    <t>MGR</t>
+  </si>
+  <si>
+    <t>Manufacture of nitrogen fertilizer</t>
+  </si>
+  <si>
+    <t>NFR</t>
+  </si>
+  <si>
+    <t>Manufacture of phosphorus fertilizer</t>
+  </si>
+  <si>
+    <t>PFR</t>
+  </si>
+  <si>
+    <t>OFR</t>
+  </si>
+  <si>
+    <t>Manufacture of potassium fertilizer</t>
+  </si>
+  <si>
+    <t>KFR</t>
+  </si>
+  <si>
+    <t>Manufacture of basic pharmaceutical products</t>
+  </si>
+  <si>
+    <t>BPH</t>
+  </si>
+  <si>
+    <t>Manufacture of rubber products</t>
+  </si>
+  <si>
+    <t>RBR</t>
+  </si>
+  <si>
+    <t>RPP</t>
+  </si>
+  <si>
+    <t>Manufacture of primary plastic products</t>
+  </si>
+  <si>
+    <t>PLP</t>
+  </si>
+  <si>
+    <t>Manufacture of secondary plastic products</t>
+  </si>
+  <si>
+    <t>PLS</t>
+  </si>
+  <si>
+    <t>Recycling of plastics</t>
+  </si>
+  <si>
+    <t>PLR</t>
+  </si>
+  <si>
+    <t>RECYCLE</t>
+  </si>
+  <si>
+    <t>Manufacture of traditional cement</t>
+  </si>
+  <si>
+    <t>CEM</t>
+  </si>
+  <si>
+    <t>NMM</t>
+  </si>
+  <si>
+    <t>CEMNT</t>
+  </si>
+  <si>
+    <t>Manufacture of cement with CCS</t>
+  </si>
+  <si>
+    <t>CMS</t>
+  </si>
+  <si>
+    <t>Manufacture of other non metallic minerals</t>
+  </si>
+  <si>
+    <t>NMX</t>
+  </si>
+  <si>
+    <t>Manufacture of steel via BF-BOF with coke injection</t>
+  </si>
+  <si>
+    <t>SCI</t>
+  </si>
+  <si>
+    <t>I_S</t>
+  </si>
+  <si>
+    <t>XIS</t>
+  </si>
+  <si>
+    <t>Manufacture of steel via BF-BOF with natural gas injection</t>
+  </si>
+  <si>
+    <t>SGI</t>
+  </si>
+  <si>
+    <t>Manufacture of steel via BF-BOF with hydrogen injection</t>
+  </si>
+  <si>
+    <t>SHI</t>
+  </si>
+  <si>
+    <t>Manufacture of steel via direct reduction with natural gas</t>
+  </si>
+  <si>
+    <t>SDG</t>
+  </si>
+  <si>
+    <t>Manufacture of steel via direct reduction with hydrogen</t>
+  </si>
+  <si>
+    <t>SDH</t>
+  </si>
+  <si>
+    <t>Manufacture of other iron and steel</t>
+  </si>
+  <si>
+    <t>Manufacture of secondary iron and steel</t>
+  </si>
+  <si>
+    <t>ISS</t>
+  </si>
+  <si>
+    <t>Recycling of iron and steel</t>
+  </si>
+  <si>
+    <t>RIS</t>
+  </si>
+  <si>
+    <t>Casting of other non-ferrous metals</t>
+  </si>
+  <si>
+    <t>NFC</t>
+  </si>
+  <si>
+    <t>NFM</t>
+  </si>
+  <si>
+    <t>ISC_NFC</t>
+  </si>
+  <si>
+    <t>Manufacture of primary aluminum</t>
+  </si>
+  <si>
+    <t>APP</t>
+  </si>
+  <si>
+    <t>Manufacture of secondary aluminum</t>
+  </si>
+  <si>
+    <t>APS</t>
+  </si>
+  <si>
+    <t>Recycling of aluminum</t>
+  </si>
+  <si>
+    <t>RAL</t>
+  </si>
+  <si>
+    <t>Manufacture of primary copper</t>
+  </si>
+  <si>
+    <t>CPP</t>
+  </si>
+  <si>
+    <t>Manufacture of secondary copper</t>
+  </si>
+  <si>
+    <t>CPS</t>
+  </si>
+  <si>
+    <t>Recycling of copper</t>
+  </si>
+  <si>
+    <t>RCP</t>
+  </si>
+  <si>
+    <t>Manufacture of magnesium: unwrought, articles</t>
+  </si>
+  <si>
+    <t>MUN</t>
+  </si>
+  <si>
+    <t>MPPR</t>
+  </si>
+  <si>
+    <t>Manufacture of semi-manufactured platinum group metals</t>
+  </si>
+  <si>
+    <t>PGR</t>
+  </si>
+  <si>
+    <t>MPR</t>
+  </si>
+  <si>
+    <t>Manufacture of refined silver</t>
+  </si>
+  <si>
+    <t>SIR</t>
+  </si>
+  <si>
+    <t>Manufacture of other metals (primary, secondary and recycling)</t>
+  </si>
+  <si>
+    <t>NFX</t>
+  </si>
+  <si>
+    <t>Manufacture of fabricated metal products</t>
+  </si>
+  <si>
+    <t>FMP</t>
+  </si>
+  <si>
+    <t>Manufacture of computer, electronic and optical products</t>
+  </si>
+  <si>
+    <t>XEL</t>
+  </si>
+  <si>
+    <t>ELE</t>
+  </si>
+  <si>
+    <t>Manufacture of solar panels</t>
+  </si>
+  <si>
+    <t>SOP</t>
+  </si>
+  <si>
+    <t>Manufacture of other electrical equipment</t>
+  </si>
+  <si>
+    <t>XEQ</t>
+  </si>
+  <si>
+    <t>EEQ</t>
+  </si>
+  <si>
+    <t>Manufacture of NCM batteries</t>
+  </si>
+  <si>
+    <t>NCM</t>
+  </si>
+  <si>
+    <t>Manufacture of NCA batteries</t>
+  </si>
+  <si>
+    <t>NCA</t>
+  </si>
+  <si>
+    <t>Manufacture of LFP batteries</t>
+  </si>
+  <si>
+    <t>LFP</t>
+  </si>
+  <si>
+    <t>Manufacture of other machinery and equipment</t>
+  </si>
+  <si>
+    <t>OME</t>
+  </si>
+  <si>
+    <t>Manufacture of wind turbines</t>
+  </si>
+  <si>
+    <t>WNT</t>
+  </si>
+  <si>
+    <t>Manufacture of electrolyzers</t>
+  </si>
+  <si>
+    <t>ELZ</t>
+  </si>
+  <si>
+    <t>Manufacture of rest of motor vehicles and parts</t>
+  </si>
+  <si>
+    <t>XMV</t>
+  </si>
+  <si>
+    <t>MVH</t>
+  </si>
+  <si>
+    <t>Manufacture of heavy duty ICEV</t>
+  </si>
+  <si>
+    <t>ICH</t>
+  </si>
+  <si>
+    <t>Manufacture of heavy duty BEV</t>
+  </si>
+  <si>
+    <t>BVH</t>
+  </si>
+  <si>
+    <t>Manufacture of heavy duty FCEV</t>
+  </si>
+  <si>
+    <t>FCH</t>
+  </si>
+  <si>
+    <t>Manufacture of light duty ICEV</t>
+  </si>
+  <si>
+    <t>ICL</t>
+  </si>
+  <si>
+    <t>Manufacture of light duty HEV</t>
+  </si>
+  <si>
+    <t>HEL</t>
+  </si>
+  <si>
+    <t>Manufacture of light duty BEV</t>
+  </si>
+  <si>
+    <t>BVL</t>
+  </si>
+  <si>
+    <t>Manufacture of rest of transport equipment</t>
+  </si>
+  <si>
+    <t>OTN</t>
+  </si>
+  <si>
+    <t>Other manufacturing</t>
+  </si>
+  <si>
+    <t>OMF</t>
+  </si>
+  <si>
+    <t>Production of electricity by coal power baseload</t>
+  </si>
+  <si>
+    <t>CoalBL</t>
+  </si>
+  <si>
+    <t>ELY</t>
+  </si>
+  <si>
+    <t>Production of electricity by gas power baseload</t>
+  </si>
+  <si>
+    <t>GasBL</t>
+  </si>
+  <si>
+    <t>Production of electricity by gas power peakload</t>
+  </si>
+  <si>
+    <t>GasP</t>
+  </si>
+  <si>
+    <t>Production of electricity by hydro power baseload</t>
+  </si>
+  <si>
+    <t>HydroBL</t>
+  </si>
+  <si>
+    <t>Production of electricity by hydro power peakload</t>
+  </si>
+  <si>
+    <t>HydroP</t>
+  </si>
+  <si>
+    <t>Production of electricity by nuclear power</t>
+  </si>
+  <si>
+    <t>NuclearBL</t>
+  </si>
+  <si>
+    <t>Production of electricity by other baseload</t>
+  </si>
+  <si>
+    <t>OtherBL</t>
+  </si>
+  <si>
+    <t>Production of electricity by oil power baseload</t>
+  </si>
+  <si>
+    <t>OilBL</t>
+  </si>
+  <si>
+    <t>Production of electricity by oil power peakload</t>
+  </si>
+  <si>
+    <t>OilP</t>
+  </si>
+  <si>
+    <t>Production of electricity by solar power</t>
+  </si>
+  <si>
+    <t>SolarP</t>
+  </si>
+  <si>
+    <t>Production of electricity by wind power</t>
+  </si>
+  <si>
+    <t>WindBL</t>
+  </si>
+  <si>
+    <t>Electricity transmission and distribution</t>
+  </si>
+  <si>
+    <t>TnD</t>
+  </si>
+  <si>
+    <t>Gas manufacture and distribution</t>
+  </si>
+  <si>
+    <t>GDT</t>
+  </si>
+  <si>
+    <t>Water and management and recycling</t>
+  </si>
+  <si>
+    <t>WTR</t>
+  </si>
+  <si>
+    <t>Construction</t>
+  </si>
+  <si>
+    <t>CNS</t>
+  </si>
+  <si>
+    <t>Trade</t>
+  </si>
+  <si>
+    <t>TRD</t>
+  </si>
+  <si>
+    <t>Accommodation, Food and service activities</t>
+  </si>
+  <si>
+    <t>AFS</t>
+  </si>
+  <si>
+    <t>Other land transport</t>
+  </si>
+  <si>
+    <t>XTP</t>
+  </si>
+  <si>
+    <t>OTP</t>
+  </si>
+  <si>
+    <t>Transport via pipeline service</t>
+  </si>
+  <si>
+    <t>TVP</t>
+  </si>
+  <si>
+    <t>Passenger road transport service</t>
+  </si>
+  <si>
+    <t>PSR</t>
+  </si>
+  <si>
+    <t>Freight road transport service</t>
+  </si>
+  <si>
+    <t>FRT</t>
+  </si>
+  <si>
+    <t>Freight international shipping service</t>
+  </si>
+  <si>
+    <t>WTP</t>
+  </si>
+  <si>
+    <t>Freight national shipping service</t>
+  </si>
+  <si>
+    <t>Passenger water transport service</t>
+  </si>
+  <si>
+    <t>Air transport service</t>
+  </si>
+  <si>
+    <t>ATP</t>
+  </si>
+  <si>
+    <t>Warehousing and support activities</t>
+  </si>
+  <si>
+    <t>WHS</t>
+  </si>
+  <si>
+    <t>Communication</t>
+  </si>
+  <si>
+    <t>CMN</t>
+  </si>
+  <si>
+    <t>Financial services nec</t>
+  </si>
+  <si>
+    <t>OFI</t>
+  </si>
+  <si>
+    <t>Insurance services</t>
+  </si>
+  <si>
+    <t>INS</t>
+  </si>
+  <si>
+    <t>Real estate activities</t>
+  </si>
+  <si>
+    <t>RSA</t>
+  </si>
+  <si>
+    <t>Business services</t>
+  </si>
+  <si>
+    <t>OBS</t>
+  </si>
+  <si>
+    <t>Recreational and other services</t>
+  </si>
+  <si>
+    <t>ROS</t>
+  </si>
+  <si>
+    <t>Public Administration and defense</t>
+  </si>
+  <si>
+    <t>OSG</t>
+  </si>
+  <si>
+    <t>Education</t>
+  </si>
+  <si>
+    <t>EDU</t>
+  </si>
+  <si>
+    <t>Human health and social work activities</t>
+  </si>
+  <si>
+    <t>HHT</t>
+  </si>
+  <si>
+    <t>Dwellings imputed rents</t>
+  </si>
+  <si>
+    <t>DWE</t>
+  </si>
+  <si>
+    <t>LCO</t>
+  </si>
+  <si>
+    <t>LMO</t>
+  </si>
+  <si>
+    <t>Permanent magnets</t>
+  </si>
+  <si>
+    <t>MAG</t>
+  </si>
+  <si>
+    <t>Manufacture of metallurgical silicon</t>
+  </si>
+  <si>
+    <t>MSI</t>
+  </si>
+  <si>
+    <t>Land</t>
+  </si>
+  <si>
+    <t>Capital</t>
+  </si>
+  <si>
+    <t>LDNRENT</t>
+  </si>
+  <si>
+    <t>FIXCAP</t>
+  </si>
+  <si>
+    <t>Natural Resources</t>
+  </si>
+  <si>
+    <t>RESRENT</t>
+  </si>
+  <si>
+    <t>Technical and professional workers</t>
+  </si>
+  <si>
+    <t>Labor</t>
+  </si>
+  <si>
+    <t>LABHSKL</t>
+  </si>
+  <si>
+    <t>Clerical workers</t>
+  </si>
+  <si>
+    <t>LABMSKL</t>
+  </si>
+  <si>
+    <t>Service shop</t>
+  </si>
+  <si>
+    <t>LABLSKL</t>
+  </si>
+  <si>
+    <t>Management</t>
+  </si>
+  <si>
+    <t>Agriculture and other low-skill workers</t>
+  </si>
+  <si>
+    <t>Taxes on production on activities by destination commodity</t>
+  </si>
+  <si>
+    <t>Tax</t>
+  </si>
+  <si>
+    <t>PRODTAX</t>
+  </si>
+  <si>
+    <t>End-user taxes on domestic purchases: purchaser – basic price</t>
+  </si>
+  <si>
+    <t>OTHTAX</t>
+  </si>
+  <si>
+    <t>End-user taxes on imported purchases: purchaser – basic price</t>
+  </si>
+  <si>
+    <t>Export taxes: VFOB - VXSB</t>
+  </si>
+  <si>
+    <t>Import taxes: VMSBA - VCIFA</t>
+  </si>
+  <si>
+    <t>International trade and transport margins</t>
+  </si>
+  <si>
+    <t>TTM</t>
+  </si>
+  <si>
+    <t>Manufacture of coke</t>
+  </si>
+  <si>
+    <t>Manufacture of LCO batteries</t>
+  </si>
+  <si>
+    <t>Manufacture of LMO batteries</t>
+  </si>
+  <si>
+    <t>Mining of natural calcium phosphates, natural aluminium calcium phosphates and phosphatic chalk</t>
+  </si>
+  <si>
     <t>Mining of natural calcium phosphates, natural aluminium calcium phosphates and phosphatic chalk: ground + unground</t>
   </si>
   <si>
-    <t>CPH</t>
-  </si>
-  <si>
-    <t>Mining of natural magnesium carbonate "magnesite"+magnesia, fused or dead-burned (sintered)</t>
-  </si>
-  <si>
-    <t>MGC</t>
-  </si>
-  <si>
-    <t>Manufacture of bovine meat products</t>
-  </si>
-  <si>
-    <t>CMT</t>
-  </si>
-  <si>
-    <t>Manufacture of meat products nec</t>
-  </si>
-  <si>
-    <t>Manufacture of vegetable oils and fats</t>
-  </si>
-  <si>
-    <t>VOL</t>
-  </si>
-  <si>
-    <t>Manufacture of dairy products</t>
-  </si>
-  <si>
-    <t>MIL</t>
-  </si>
-  <si>
-    <t>Manufacture of processed rice</t>
-  </si>
-  <si>
-    <t>PCR</t>
-  </si>
-  <si>
-    <t>Manufacture of sugar</t>
-  </si>
-  <si>
-    <t>SGR</t>
-  </si>
-  <si>
-    <t>Manufacture of food products nec</t>
-  </si>
-  <si>
-    <t>OFD</t>
-  </si>
-  <si>
-    <t>Manufacture of beverages and tobacco products</t>
-  </si>
-  <si>
-    <t>B_T</t>
-  </si>
-  <si>
-    <t>Manufacture of textiles</t>
-  </si>
-  <si>
-    <t>TEX</t>
-  </si>
-  <si>
-    <t>Manufacture of wearing apparel</t>
-  </si>
-  <si>
-    <t>WAP</t>
-  </si>
-  <si>
-    <t>Manufacture of leather products</t>
-  </si>
-  <si>
-    <t>LEA</t>
-  </si>
-  <si>
-    <t>Manufacture of wood products</t>
-  </si>
-  <si>
-    <t>LUM</t>
-  </si>
-  <si>
-    <t>Manufacture of paper products, publishing</t>
-  </si>
-  <si>
-    <t>PPP</t>
-  </si>
-  <si>
-    <t>Manufacture of petroleum products</t>
-  </si>
-  <si>
-    <t>PEP</t>
-  </si>
-  <si>
-    <t>P_C</t>
-  </si>
-  <si>
-    <t>PCP</t>
-  </si>
-  <si>
-    <t>Manufacture of coal products</t>
-  </si>
-  <si>
-    <t>Manufacture of other chemicals</t>
-  </si>
-  <si>
-    <t>XCH</t>
-  </si>
-  <si>
-    <t>CHM</t>
-  </si>
-  <si>
-    <t>XCH_BPH</t>
-  </si>
-  <si>
-    <t>Manufacture of ammonia</t>
-  </si>
-  <si>
-    <t>AMM</t>
-  </si>
-  <si>
-    <t>Manufacture of hydrogen via electrolysis</t>
-  </si>
-  <si>
-    <t>HYE</t>
-  </si>
-  <si>
-    <t>Manufacture of hydrogen via steam reforming</t>
-  </si>
-  <si>
-    <t>HYS</t>
-  </si>
-  <si>
-    <t>Manufacture of methanol</t>
-  </si>
-  <si>
-    <t>MTH</t>
-  </si>
-  <si>
-    <t>Manufacture of high value chemicals</t>
-  </si>
-  <si>
-    <t>HVC</t>
-  </si>
-  <si>
-    <t>Manufacture of artificial graphite</t>
-  </si>
-  <si>
-    <t>AGT</t>
-  </si>
-  <si>
-    <t>Manufacture of refined lithium</t>
-  </si>
-  <si>
-    <t>LIR</t>
-  </si>
-  <si>
-    <t>Manufacture of refined rare earths</t>
-  </si>
-  <si>
-    <t>RER</t>
-  </si>
-  <si>
-    <t>Manufacture of refined manganese</t>
-  </si>
-  <si>
-    <t>MNR</t>
-  </si>
-  <si>
-    <t>Manufacture of refined nickel</t>
-  </si>
-  <si>
-    <t>NIR</t>
-  </si>
-  <si>
-    <t>Manufacture of refined cobalt</t>
-  </si>
-  <si>
-    <t>COR</t>
-  </si>
-  <si>
-    <t>Manufacture of refined zinc</t>
-  </si>
-  <si>
-    <t>ZIR</t>
-  </si>
-  <si>
-    <t>LZR</t>
-  </si>
-  <si>
-    <t>Manufacture of refined chromium</t>
-  </si>
-  <si>
-    <t>CRR</t>
-  </si>
-  <si>
-    <t>Manufacture of refined titanium</t>
-  </si>
-  <si>
-    <t>TIR</t>
-  </si>
-  <si>
-    <t>Manufacture of refined gallium</t>
-  </si>
-  <si>
-    <t>GAR</t>
-  </si>
-  <si>
-    <t>Manufacture of refined magnesium</t>
-  </si>
-  <si>
-    <t>MGR</t>
-  </si>
-  <si>
-    <t>Manufacture of nitrogen fertilizer</t>
-  </si>
-  <si>
-    <t>NFR</t>
-  </si>
-  <si>
-    <t>Manufacture of phosphorus fertilizer</t>
-  </si>
-  <si>
-    <t>PFR</t>
-  </si>
-  <si>
-    <t>OFR</t>
-  </si>
-  <si>
-    <t>Manufacture of potassium fertilizer</t>
-  </si>
-  <si>
-    <t>KFR</t>
-  </si>
-  <si>
-    <t>Manufacture of basic pharmaceutical products</t>
-  </si>
-  <si>
-    <t>BPH</t>
-  </si>
-  <si>
-    <t>Manufacture of rubber products</t>
-  </si>
-  <si>
-    <t>RBR</t>
-  </si>
-  <si>
-    <t>RPP</t>
-  </si>
-  <si>
-    <t>Manufacture of primary plastic products</t>
-  </si>
-  <si>
-    <t>PLP</t>
-  </si>
-  <si>
-    <t>Manufacture of secondary plastic products</t>
-  </si>
-  <si>
-    <t>PLS</t>
-  </si>
-  <si>
-    <t>Recycling of plastics</t>
-  </si>
-  <si>
-    <t>PLR</t>
-  </si>
-  <si>
-    <t>RECYCLE</t>
-  </si>
-  <si>
-    <t>Manufacture of traditional cement</t>
-  </si>
-  <si>
-    <t>CEM</t>
-  </si>
-  <si>
-    <t>NMM</t>
-  </si>
-  <si>
-    <t>CEMNT</t>
-  </si>
-  <si>
-    <t>Manufacture of cement with CCS</t>
-  </si>
-  <si>
-    <t>CMS</t>
-  </si>
-  <si>
-    <t>Manufacture of other non metallic minerals</t>
-  </si>
-  <si>
-    <t>NMX</t>
-  </si>
-  <si>
-    <t>Manufacture of steel via BF-BOF with coke injection</t>
-  </si>
-  <si>
-    <t>SCI</t>
-  </si>
-  <si>
-    <t>I_S</t>
-  </si>
-  <si>
-    <t>XIS</t>
-  </si>
-  <si>
-    <t>Manufacture of steel via BF-BOF with natural gas injection</t>
-  </si>
-  <si>
-    <t>SGI</t>
-  </si>
-  <si>
-    <t>Manufacture of steel via BF-BOF with hydrogen injection</t>
-  </si>
-  <si>
-    <t>SHI</t>
-  </si>
-  <si>
-    <t>Manufacture of steel via direct reduction with natural gas</t>
-  </si>
-  <si>
-    <t>SDG</t>
-  </si>
-  <si>
-    <t>Manufacture of steel via direct reduction with hydrogen</t>
-  </si>
-  <si>
-    <t>SDH</t>
-  </si>
-  <si>
-    <t>Manufacture of other iron and steel</t>
-  </si>
-  <si>
-    <t>Manufacture of secondary iron and steel</t>
-  </si>
-  <si>
-    <t>ISS</t>
-  </si>
-  <si>
-    <t>Recycling of iron and steel</t>
-  </si>
-  <si>
-    <t>RIS</t>
-  </si>
-  <si>
-    <t>Casting of other non-ferrous metals</t>
-  </si>
-  <si>
-    <t>NFC</t>
-  </si>
-  <si>
-    <t>NFM</t>
-  </si>
-  <si>
-    <t>ISC_NFC</t>
-  </si>
-  <si>
-    <t>Manufacture of primary aluminum</t>
-  </si>
-  <si>
-    <t>APP</t>
-  </si>
-  <si>
-    <t>Manufacture of secondary aluminum</t>
-  </si>
-  <si>
-    <t>APS</t>
-  </si>
-  <si>
-    <t>Recycling of aluminum</t>
-  </si>
-  <si>
-    <t>RAL</t>
-  </si>
-  <si>
-    <t>Manufacture of primary copper</t>
-  </si>
-  <si>
-    <t>CPP</t>
-  </si>
-  <si>
-    <t>Manufacture of secondary copper</t>
-  </si>
-  <si>
-    <t>CPS</t>
-  </si>
-  <si>
-    <t>Recycling of copper</t>
-  </si>
-  <si>
-    <t>RCP</t>
-  </si>
-  <si>
-    <t>Manufacture of magnesium: unwrought, articles</t>
-  </si>
-  <si>
-    <t>MUN</t>
-  </si>
-  <si>
-    <t>MPPR</t>
-  </si>
-  <si>
-    <t>Manufacture of semi-manufactured platinum group metals</t>
-  </si>
-  <si>
-    <t>PGR</t>
-  </si>
-  <si>
-    <t>MPR</t>
-  </si>
-  <si>
-    <t>Manufacture of refined silver</t>
-  </si>
-  <si>
-    <t>SIR</t>
-  </si>
-  <si>
-    <t>Manufacture of other metals (primary, secondary and recycling)</t>
-  </si>
-  <si>
-    <t>NFX</t>
-  </si>
-  <si>
-    <t>Manufacture of fabricated metal products</t>
-  </si>
-  <si>
-    <t>FMP</t>
-  </si>
-  <si>
-    <t>Manufacture of computer, electronic and optical products</t>
-  </si>
-  <si>
-    <t>XEL</t>
-  </si>
-  <si>
-    <t>ELE</t>
-  </si>
-  <si>
-    <t>Manufacture of solar panels</t>
-  </si>
-  <si>
-    <t>SOP</t>
-  </si>
-  <si>
-    <t>Manufacture of other electrical equipment</t>
-  </si>
-  <si>
-    <t>XEQ</t>
-  </si>
-  <si>
-    <t>EEQ</t>
-  </si>
-  <si>
-    <t>Manufacture of NCM batteries</t>
-  </si>
-  <si>
-    <t>NCM</t>
-  </si>
-  <si>
-    <t>Manufacture of NCA batteries</t>
-  </si>
-  <si>
-    <t>NCA</t>
-  </si>
-  <si>
-    <t>Manufacture of LFP batteries</t>
-  </si>
-  <si>
-    <t>LFP</t>
-  </si>
-  <si>
-    <t>Manufacture of other machinery and equipment</t>
-  </si>
-  <si>
-    <t>OME</t>
-  </si>
-  <si>
-    <t>Manufacture of wind turbines</t>
-  </si>
-  <si>
-    <t>WNT</t>
-  </si>
-  <si>
-    <t>Manufacture of electrolyzers</t>
-  </si>
-  <si>
-    <t>ELZ</t>
-  </si>
-  <si>
-    <t>Manufacture of rest of motor vehicles and parts</t>
-  </si>
-  <si>
-    <t>XMV</t>
-  </si>
-  <si>
-    <t>MVH</t>
-  </si>
-  <si>
-    <t>Manufacture of heavy duty ICEV</t>
-  </si>
-  <si>
-    <t>ICH</t>
-  </si>
-  <si>
-    <t>Manufacture of heavy duty BEV</t>
-  </si>
-  <si>
-    <t>BVH</t>
-  </si>
-  <si>
-    <t>Manufacture of heavy duty FCEV</t>
-  </si>
-  <si>
-    <t>FCH</t>
-  </si>
-  <si>
-    <t>Manufacture of light duty ICEV</t>
-  </si>
-  <si>
-    <t>ICL</t>
-  </si>
-  <si>
-    <t>Manufacture of light duty HEV</t>
-  </si>
-  <si>
-    <t>HEL</t>
-  </si>
-  <si>
-    <t>Manufacture of light duty BEV</t>
-  </si>
-  <si>
-    <t>BVL</t>
-  </si>
-  <si>
-    <t>Manufacture of rest of transport equipment</t>
-  </si>
-  <si>
-    <t>OTN</t>
-  </si>
-  <si>
-    <t>Other manufacturing</t>
-  </si>
-  <si>
-    <t>OMF</t>
-  </si>
-  <si>
-    <t>Production of electricity by coal power baseload</t>
-  </si>
-  <si>
-    <t>CoalBL</t>
-  </si>
-  <si>
-    <t>ELY</t>
-  </si>
-  <si>
-    <t>Production of electricity by gas power baseload</t>
-  </si>
-  <si>
-    <t>GasBL</t>
-  </si>
-  <si>
-    <t>Production of electricity by gas power peakload</t>
-  </si>
-  <si>
-    <t>GasP</t>
-  </si>
-  <si>
-    <t>Production of electricity by hydro power baseload</t>
-  </si>
-  <si>
-    <t>HydroBL</t>
-  </si>
-  <si>
-    <t>Production of electricity by hydro power peakload</t>
-  </si>
-  <si>
-    <t>HydroP</t>
-  </si>
-  <si>
-    <t>Production of electricity by nuclear power</t>
-  </si>
-  <si>
-    <t>NuclearBL</t>
-  </si>
-  <si>
-    <t>Production of electricity by other baseload</t>
-  </si>
-  <si>
-    <t>OtherBL</t>
-  </si>
-  <si>
-    <t>Production of electricity by oil power baseload</t>
-  </si>
-  <si>
-    <t>OilBL</t>
-  </si>
-  <si>
-    <t>Production of electricity by oil power peakload</t>
-  </si>
-  <si>
-    <t>OilP</t>
-  </si>
-  <si>
-    <t>Production of electricity by solar power</t>
-  </si>
-  <si>
-    <t>SolarP</t>
-  </si>
-  <si>
-    <t>Production of electricity by wind power</t>
-  </si>
-  <si>
-    <t>WindBL</t>
-  </si>
-  <si>
-    <t>Electricity transmission and distribution</t>
-  </si>
-  <si>
-    <t>TnD</t>
-  </si>
-  <si>
-    <t>Gas manufacture and distribution</t>
-  </si>
-  <si>
-    <t>GDT</t>
-  </si>
-  <si>
-    <t>Water and management and recycling</t>
-  </si>
-  <si>
-    <t>WTR</t>
-  </si>
-  <si>
-    <t>Construction</t>
-  </si>
-  <si>
-    <t>CNS</t>
-  </si>
-  <si>
-    <t>Trade</t>
-  </si>
-  <si>
-    <t>TRD</t>
-  </si>
-  <si>
-    <t>Accommodation, Food and service activities</t>
-  </si>
-  <si>
-    <t>AFS</t>
-  </si>
-  <si>
-    <t>Other land transport</t>
-  </si>
-  <si>
-    <t>XTP</t>
-  </si>
-  <si>
-    <t>OTP</t>
-  </si>
-  <si>
-    <t>Transport via pipeline service</t>
-  </si>
-  <si>
-    <t>TVP</t>
-  </si>
-  <si>
-    <t>Passenger road transport service</t>
-  </si>
-  <si>
-    <t>PSR</t>
-  </si>
-  <si>
-    <t>Freight road transport service</t>
-  </si>
-  <si>
-    <t>FRT</t>
-  </si>
-  <si>
-    <t>Freight international shipping service</t>
-  </si>
-  <si>
-    <t>WTP</t>
-  </si>
-  <si>
-    <t>Freight national shipping service</t>
-  </si>
-  <si>
-    <t>Passenger water transport service</t>
-  </si>
-  <si>
-    <t>Air transport service</t>
-  </si>
-  <si>
-    <t>ATP</t>
-  </si>
-  <si>
-    <t>Warehousing and support activities</t>
-  </si>
-  <si>
-    <t>WHS</t>
-  </si>
-  <si>
-    <t>Communication</t>
-  </si>
-  <si>
-    <t>CMN</t>
-  </si>
-  <si>
-    <t>Financial services nec</t>
-  </si>
-  <si>
-    <t>OFI</t>
-  </si>
-  <si>
-    <t>Insurance services</t>
-  </si>
-  <si>
-    <t>INS</t>
-  </si>
-  <si>
-    <t>Real estate activities</t>
-  </si>
-  <si>
-    <t>RSA</t>
-  </si>
-  <si>
-    <t>Business services</t>
-  </si>
-  <si>
-    <t>OBS</t>
-  </si>
-  <si>
-    <t>Recreational and other services</t>
-  </si>
-  <si>
-    <t>ROS</t>
-  </si>
-  <si>
-    <t>Public Administration and defense</t>
-  </si>
-  <si>
-    <t>OSG</t>
-  </si>
-  <si>
-    <t>Education</t>
-  </si>
-  <si>
-    <t>EDU</t>
-  </si>
-  <si>
-    <t>Human health and social work activities</t>
-  </si>
-  <si>
-    <t>HHT</t>
-  </si>
-  <si>
-    <t>Dwellings imputed rents</t>
-  </si>
-  <si>
-    <t>DWE</t>
-  </si>
-  <si>
-    <t>Lithium Cobalt Oxide batteries</t>
-  </si>
-  <si>
-    <t>LCO</t>
-  </si>
-  <si>
-    <t>Lithium Manganese Oxide batteries</t>
-  </si>
-  <si>
-    <t>LMO</t>
-  </si>
-  <si>
-    <t>Permanent magnets</t>
-  </si>
-  <si>
-    <t>MAG</t>
-  </si>
-  <si>
-    <t>Manufacture of metallurgical silicon</t>
-  </si>
-  <si>
-    <t>MSI</t>
-  </si>
-  <si>
-    <t>Land</t>
-  </si>
-  <si>
-    <t>Capital</t>
-  </si>
-  <si>
-    <t>LDNRENT</t>
-  </si>
-  <si>
-    <t>FIXCAP</t>
-  </si>
-  <si>
-    <t>Natural Resources</t>
-  </si>
-  <si>
-    <t>RESRENT</t>
-  </si>
-  <si>
-    <t>Technical and professional workers</t>
-  </si>
-  <si>
-    <t>Labor</t>
-  </si>
-  <si>
-    <t>LABHSKL</t>
-  </si>
-  <si>
-    <t>Clerical workers</t>
-  </si>
-  <si>
-    <t>LABMSKL</t>
-  </si>
-  <si>
-    <t>Service shop</t>
-  </si>
-  <si>
-    <t>LABLSKL</t>
-  </si>
-  <si>
-    <t>Management</t>
-  </si>
-  <si>
-    <t>Agriculture and other low-skill workers</t>
-  </si>
-  <si>
-    <t>Taxes on production on activities by destination commodity</t>
-  </si>
-  <si>
-    <t>Tax</t>
-  </si>
-  <si>
-    <t>PRODTAX</t>
-  </si>
-  <si>
-    <t>End-user taxes on domestic purchases: purchaser – basic price</t>
-  </si>
-  <si>
-    <t>OTHTAX</t>
-  </si>
-  <si>
-    <t>End-user taxes on imported purchases: purchaser – basic price</t>
-  </si>
-  <si>
-    <t>Export taxes: VFOB - VXSB</t>
-  </si>
-  <si>
-    <t>Import taxes: VMSBA - VCIFA</t>
-  </si>
-  <si>
-    <t>International trade and transport margins</t>
-  </si>
-  <si>
-    <t>TTM</t>
-  </si>
-  <si>
-    <t>Manufacture of coke</t>
+    <t>Mining of natural magnesium carbonate (magnesite) + magnesia, fused or dead-burned</t>
   </si>
 </sst>
 </file>
@@ -1738,156 +1744,156 @@
     </row>
     <row r="2" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="5" t="s">
-        <v>403</v>
+        <v>400</v>
       </c>
       <c r="B2" t="s">
-        <v>404</v>
+        <v>401</v>
       </c>
       <c r="C2" t="s">
-        <v>405</v>
+        <v>402</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="5" t="s">
-        <v>404</v>
+        <v>401</v>
       </c>
       <c r="B3" t="s">
-        <v>404</v>
+        <v>401</v>
       </c>
       <c r="C3" t="s">
-        <v>406</v>
+        <v>403</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="5" t="s">
-        <v>407</v>
+        <v>404</v>
       </c>
       <c r="B4" t="s">
-        <v>404</v>
+        <v>401</v>
       </c>
       <c r="C4" t="s">
-        <v>408</v>
+        <v>405</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="6" t="s">
-        <v>409</v>
+        <v>406</v>
       </c>
       <c r="B5" t="s">
-        <v>410</v>
+        <v>407</v>
       </c>
       <c r="C5" t="s">
-        <v>411</v>
+        <v>408</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="6" t="s">
-        <v>412</v>
+        <v>409</v>
       </c>
       <c r="B6" t="s">
+        <v>407</v>
+      </c>
+      <c r="C6" t="s">
         <v>410</v>
-      </c>
-      <c r="C6" t="s">
-        <v>413</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="6" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
       <c r="B7" t="s">
-        <v>410</v>
+        <v>407</v>
       </c>
       <c r="C7" t="s">
-        <v>415</v>
+        <v>412</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="6" t="s">
-        <v>416</v>
+        <v>413</v>
       </c>
       <c r="B8" t="s">
-        <v>410</v>
+        <v>407</v>
       </c>
       <c r="C8" t="s">
-        <v>411</v>
+        <v>408</v>
       </c>
     </row>
     <row r="9" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="6" t="s">
-        <v>417</v>
+        <v>414</v>
       </c>
       <c r="B9" t="s">
-        <v>410</v>
+        <v>407</v>
       </c>
       <c r="C9" t="s">
-        <v>415</v>
+        <v>412</v>
       </c>
     </row>
     <row r="10" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="6" t="s">
-        <v>418</v>
+        <v>415</v>
       </c>
       <c r="B10" t="s">
-        <v>419</v>
+        <v>416</v>
       </c>
       <c r="C10" t="s">
-        <v>420</v>
+        <v>417</v>
       </c>
     </row>
     <row r="11" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="6" t="s">
-        <v>421</v>
+        <v>418</v>
       </c>
       <c r="B11" t="s">
+        <v>416</v>
+      </c>
+      <c r="C11" t="s">
         <v>419</v>
-      </c>
-      <c r="C11" t="s">
-        <v>422</v>
       </c>
     </row>
     <row r="12" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="6" t="s">
-        <v>423</v>
+        <v>420</v>
       </c>
       <c r="B12" t="s">
+        <v>416</v>
+      </c>
+      <c r="C12" t="s">
         <v>419</v>
-      </c>
-      <c r="C12" t="s">
-        <v>422</v>
       </c>
     </row>
     <row r="13" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="6" t="s">
-        <v>424</v>
+        <v>421</v>
       </c>
       <c r="B13" t="s">
+        <v>416</v>
+      </c>
+      <c r="C13" t="s">
         <v>419</v>
-      </c>
-      <c r="C13" t="s">
-        <v>422</v>
       </c>
     </row>
     <row r="14" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="6" t="s">
-        <v>425</v>
+        <v>422</v>
       </c>
       <c r="B14" t="s">
+        <v>416</v>
+      </c>
+      <c r="C14" t="s">
         <v>419</v>
-      </c>
-      <c r="C14" t="s">
-        <v>422</v>
       </c>
     </row>
     <row r="15" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="4" t="s">
-        <v>426</v>
+        <v>423</v>
       </c>
       <c r="B15" t="s">
-        <v>427</v>
+        <v>424</v>
       </c>
       <c r="C15" t="s">
-        <v>422</v>
+        <v>419</v>
       </c>
     </row>
   </sheetData>
@@ -1900,7 +1906,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:E189"/>
+  <dimension ref="A1:E191"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="102.33203125" bestFit="1" customWidth="1"/>
@@ -2873,10 +2879,10 @@
     </row>
     <row r="66" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
+        <v>429</v>
+      </c>
+      <c r="B66" t="s">
         <v>141</v>
-      </c>
-      <c r="B66" t="s">
-        <v>142</v>
       </c>
       <c r="C66" t="s">
         <v>100</v>
@@ -2887,10 +2893,10 @@
     </row>
     <row r="67" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
-        <v>143</v>
+        <v>428</v>
       </c>
       <c r="B67" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="C67" t="s">
         <v>100</v>
@@ -2898,350 +2904,347 @@
       <c r="D67" t="s">
         <v>101</v>
       </c>
-      <c r="E67" t="s">
-        <v>109</v>
-      </c>
     </row>
     <row r="68" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="B68" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="C68" t="s">
-        <v>146</v>
+        <v>100</v>
       </c>
       <c r="D68" t="s">
-        <v>146</v>
+        <v>101</v>
+      </c>
+      <c r="E68" t="s">
+        <v>109</v>
       </c>
     </row>
     <row r="69" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
-        <v>147</v>
+        <v>430</v>
       </c>
       <c r="B69" t="s">
-        <v>135</v>
+        <v>143</v>
       </c>
       <c r="C69" t="s">
-        <v>135</v>
+        <v>100</v>
       </c>
       <c r="D69" t="s">
-        <v>135</v>
+        <v>101</v>
+      </c>
+      <c r="E69" t="s">
+        <v>109</v>
       </c>
     </row>
     <row r="70" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="B70" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="C70" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="D70" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
     </row>
     <row r="71" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="B71" t="s">
-        <v>151</v>
+        <v>135</v>
       </c>
       <c r="C71" t="s">
-        <v>151</v>
+        <v>135</v>
       </c>
       <c r="D71" t="s">
-        <v>151</v>
+        <v>135</v>
       </c>
     </row>
     <row r="72" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
-        <v>152</v>
+        <v>147</v>
       </c>
       <c r="B72" t="s">
-        <v>153</v>
+        <v>148</v>
       </c>
       <c r="C72" t="s">
-        <v>153</v>
+        <v>148</v>
       </c>
       <c r="D72" t="s">
-        <v>153</v>
+        <v>148</v>
       </c>
     </row>
     <row r="73" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
-        <v>154</v>
+        <v>149</v>
       </c>
       <c r="B73" t="s">
-        <v>155</v>
+        <v>150</v>
       </c>
       <c r="C73" t="s">
-        <v>155</v>
+        <v>150</v>
       </c>
       <c r="D73" t="s">
-        <v>155</v>
+        <v>150</v>
       </c>
     </row>
     <row r="74" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
-        <v>156</v>
+        <v>151</v>
       </c>
       <c r="B74" t="s">
-        <v>157</v>
+        <v>152</v>
       </c>
       <c r="C74" t="s">
-        <v>157</v>
+        <v>152</v>
       </c>
       <c r="D74" t="s">
-        <v>157</v>
+        <v>152</v>
       </c>
     </row>
     <row r="75" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A75" t="s">
-        <v>158</v>
+        <v>153</v>
       </c>
       <c r="B75" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
       <c r="C75" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
       <c r="D75" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
     </row>
     <row r="76" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
-        <v>160</v>
+        <v>155</v>
       </c>
       <c r="B76" t="s">
-        <v>161</v>
+        <v>156</v>
       </c>
       <c r="C76" t="s">
-        <v>161</v>
+        <v>156</v>
       </c>
       <c r="D76" t="s">
-        <v>161</v>
+        <v>156</v>
       </c>
     </row>
     <row r="77" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
-        <v>162</v>
+        <v>157</v>
       </c>
       <c r="B77" t="s">
-        <v>163</v>
+        <v>158</v>
       </c>
       <c r="C77" t="s">
-        <v>163</v>
+        <v>158</v>
       </c>
       <c r="D77" t="s">
-        <v>163</v>
+        <v>158</v>
       </c>
     </row>
     <row r="78" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A78" t="s">
-        <v>164</v>
+        <v>159</v>
       </c>
       <c r="B78" t="s">
-        <v>165</v>
+        <v>160</v>
       </c>
       <c r="C78" t="s">
-        <v>165</v>
+        <v>160</v>
       </c>
       <c r="D78" t="s">
-        <v>165</v>
+        <v>160</v>
       </c>
     </row>
     <row r="79" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A79" t="s">
-        <v>166</v>
+        <v>161</v>
       </c>
       <c r="B79" t="s">
-        <v>167</v>
+        <v>162</v>
       </c>
       <c r="C79" t="s">
-        <v>167</v>
+        <v>162</v>
       </c>
       <c r="D79" t="s">
-        <v>167</v>
+        <v>162</v>
       </c>
     </row>
     <row r="80" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A80" t="s">
-        <v>168</v>
+        <v>163</v>
       </c>
       <c r="B80" t="s">
-        <v>169</v>
+        <v>164</v>
       </c>
       <c r="C80" t="s">
-        <v>169</v>
+        <v>164</v>
       </c>
       <c r="D80" t="s">
-        <v>169</v>
+        <v>164</v>
       </c>
     </row>
     <row r="81" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A81" t="s">
-        <v>170</v>
+        <v>165</v>
       </c>
       <c r="B81" t="s">
-        <v>171</v>
+        <v>166</v>
       </c>
       <c r="C81" t="s">
-        <v>172</v>
+        <v>166</v>
       </c>
       <c r="D81" t="s">
-        <v>173</v>
+        <v>166</v>
       </c>
     </row>
     <row r="82" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A82" t="s">
-        <v>174</v>
+        <v>167</v>
       </c>
       <c r="B82" t="s">
-        <v>173</v>
+        <v>168</v>
       </c>
       <c r="C82" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="D82" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
     </row>
     <row r="83" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A83" t="s">
-        <v>175</v>
+        <v>169</v>
       </c>
       <c r="B83" t="s">
-        <v>176</v>
+        <v>170</v>
       </c>
       <c r="C83" t="s">
-        <v>177</v>
+        <v>171</v>
       </c>
       <c r="D83" t="s">
-        <v>178</v>
+        <v>172</v>
       </c>
     </row>
     <row r="84" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A84" t="s">
-        <v>179</v>
+        <v>173</v>
       </c>
       <c r="B84" t="s">
-        <v>180</v>
+        <v>172</v>
       </c>
       <c r="C84" t="s">
-        <v>177</v>
+        <v>171</v>
       </c>
       <c r="D84" t="s">
-        <v>178</v>
+        <v>170</v>
       </c>
     </row>
     <row r="85" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A85" t="s">
-        <v>181</v>
+        <v>174</v>
       </c>
       <c r="B85" t="s">
-        <v>182</v>
+        <v>175</v>
       </c>
       <c r="C85" t="s">
+        <v>176</v>
+      </c>
+      <c r="D85" t="s">
         <v>177</v>
-      </c>
-      <c r="D85" t="s">
-        <v>178</v>
       </c>
     </row>
     <row r="86" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A86" t="s">
-        <v>183</v>
+        <v>178</v>
       </c>
       <c r="B86" t="s">
-        <v>184</v>
+        <v>179</v>
       </c>
       <c r="C86" t="s">
+        <v>176</v>
+      </c>
+      <c r="D86" t="s">
         <v>177</v>
-      </c>
-      <c r="D86" t="s">
-        <v>178</v>
       </c>
     </row>
     <row r="87" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A87" t="s">
-        <v>185</v>
+        <v>180</v>
       </c>
       <c r="B87" t="s">
-        <v>186</v>
+        <v>181</v>
       </c>
       <c r="C87" t="s">
+        <v>176</v>
+      </c>
+      <c r="D87" t="s">
         <v>177</v>
-      </c>
-      <c r="D87" t="s">
-        <v>178</v>
       </c>
     </row>
     <row r="88" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A88" t="s">
-        <v>187</v>
+        <v>182</v>
       </c>
       <c r="B88" t="s">
-        <v>188</v>
+        <v>183</v>
       </c>
       <c r="C88" t="s">
+        <v>176</v>
+      </c>
+      <c r="D88" t="s">
         <v>177</v>
-      </c>
-      <c r="D88" t="s">
-        <v>178</v>
       </c>
     </row>
     <row r="89" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A89" t="s">
-        <v>189</v>
+        <v>184</v>
       </c>
       <c r="B89" t="s">
-        <v>190</v>
+        <v>185</v>
       </c>
       <c r="C89" t="s">
+        <v>176</v>
+      </c>
+      <c r="D89" t="s">
         <v>177</v>
-      </c>
-      <c r="D89" t="s">
-        <v>178</v>
-      </c>
-      <c r="E89" t="s">
-        <v>109</v>
       </c>
     </row>
     <row r="90" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A90" t="s">
-        <v>191</v>
+        <v>186</v>
       </c>
       <c r="B90" t="s">
-        <v>192</v>
+        <v>187</v>
       </c>
       <c r="C90" t="s">
+        <v>176</v>
+      </c>
+      <c r="D90" t="s">
         <v>177</v>
-      </c>
-      <c r="D90" t="s">
-        <v>178</v>
-      </c>
-      <c r="E90" t="s">
-        <v>109</v>
       </c>
     </row>
     <row r="91" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A91" t="s">
-        <v>193</v>
+        <v>188</v>
       </c>
       <c r="B91" t="s">
-        <v>194</v>
+        <v>189</v>
       </c>
       <c r="C91" t="s">
+        <v>176</v>
+      </c>
+      <c r="D91" t="s">
         <v>177</v>
-      </c>
-      <c r="D91" t="s">
-        <v>178</v>
       </c>
       <c r="E91" t="s">
         <v>109</v>
@@ -3249,16 +3252,16 @@
     </row>
     <row r="92" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A92" t="s">
-        <v>195</v>
+        <v>190</v>
       </c>
       <c r="B92" t="s">
-        <v>196</v>
+        <v>191</v>
       </c>
       <c r="C92" t="s">
+        <v>176</v>
+      </c>
+      <c r="D92" t="s">
         <v>177</v>
-      </c>
-      <c r="D92" t="s">
-        <v>178</v>
       </c>
       <c r="E92" t="s">
         <v>109</v>
@@ -3266,16 +3269,16 @@
     </row>
     <row r="93" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A93" t="s">
-        <v>197</v>
+        <v>192</v>
       </c>
       <c r="B93" t="s">
-        <v>198</v>
+        <v>193</v>
       </c>
       <c r="C93" t="s">
+        <v>176</v>
+      </c>
+      <c r="D93" t="s">
         <v>177</v>
-      </c>
-      <c r="D93" t="s">
-        <v>178</v>
       </c>
       <c r="E93" t="s">
         <v>109</v>
@@ -3283,16 +3286,16 @@
     </row>
     <row r="94" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A94" t="s">
-        <v>199</v>
+        <v>194</v>
       </c>
       <c r="B94" t="s">
-        <v>200</v>
+        <v>195</v>
       </c>
       <c r="C94" t="s">
+        <v>176</v>
+      </c>
+      <c r="D94" t="s">
         <v>177</v>
-      </c>
-      <c r="D94" t="s">
-        <v>178</v>
       </c>
       <c r="E94" t="s">
         <v>109</v>
@@ -3300,16 +3303,16 @@
     </row>
     <row r="95" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A95" t="s">
-        <v>201</v>
+        <v>196</v>
       </c>
       <c r="B95" t="s">
-        <v>202</v>
+        <v>197</v>
       </c>
       <c r="C95" t="s">
+        <v>176</v>
+      </c>
+      <c r="D95" t="s">
         <v>177</v>
-      </c>
-      <c r="D95" t="s">
-        <v>203</v>
       </c>
       <c r="E95" t="s">
         <v>109</v>
@@ -3317,16 +3320,16 @@
     </row>
     <row r="96" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A96" t="s">
-        <v>204</v>
+        <v>198</v>
       </c>
       <c r="B96" t="s">
-        <v>205</v>
+        <v>199</v>
       </c>
       <c r="C96" t="s">
+        <v>176</v>
+      </c>
+      <c r="D96" t="s">
         <v>177</v>
-      </c>
-      <c r="D96" t="s">
-        <v>178</v>
       </c>
       <c r="E96" t="s">
         <v>109</v>
@@ -3334,16 +3337,16 @@
     </row>
     <row r="97" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A97" t="s">
-        <v>206</v>
+        <v>200</v>
       </c>
       <c r="B97" t="s">
-        <v>207</v>
+        <v>201</v>
       </c>
       <c r="C97" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="D97" t="s">
-        <v>178</v>
+        <v>202</v>
       </c>
       <c r="E97" t="s">
         <v>109</v>
@@ -3351,16 +3354,16 @@
     </row>
     <row r="98" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A98" t="s">
-        <v>208</v>
+        <v>203</v>
       </c>
       <c r="B98" t="s">
-        <v>209</v>
+        <v>204</v>
       </c>
       <c r="C98" t="s">
+        <v>176</v>
+      </c>
+      <c r="D98" t="s">
         <v>177</v>
-      </c>
-      <c r="D98" t="s">
-        <v>178</v>
       </c>
       <c r="E98" t="s">
         <v>109</v>
@@ -3368,30 +3371,33 @@
     </row>
     <row r="99" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A99" t="s">
-        <v>210</v>
+        <v>205</v>
       </c>
       <c r="B99" t="s">
-        <v>211</v>
+        <v>206</v>
       </c>
       <c r="C99" t="s">
+        <v>176</v>
+      </c>
+      <c r="D99" t="s">
         <v>177</v>
       </c>
-      <c r="D99" t="s">
-        <v>178</v>
+      <c r="E99" t="s">
+        <v>109</v>
       </c>
     </row>
     <row r="100" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A100" t="s">
-        <v>212</v>
+        <v>207</v>
       </c>
       <c r="B100" t="s">
-        <v>213</v>
+        <v>208</v>
       </c>
       <c r="C100" t="s">
+        <v>176</v>
+      </c>
+      <c r="D100" t="s">
         <v>177</v>
-      </c>
-      <c r="D100" t="s">
-        <v>213</v>
       </c>
       <c r="E100" t="s">
         <v>109</v>
@@ -3399,33 +3405,30 @@
     </row>
     <row r="101" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A101" t="s">
-        <v>214</v>
+        <v>209</v>
       </c>
       <c r="B101" t="s">
-        <v>215</v>
+        <v>210</v>
       </c>
       <c r="C101" t="s">
+        <v>176</v>
+      </c>
+      <c r="D101" t="s">
         <v>177</v>
-      </c>
-      <c r="D101" t="s">
-        <v>216</v>
-      </c>
-      <c r="E101" t="s">
-        <v>109</v>
       </c>
     </row>
     <row r="102" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A102" t="s">
-        <v>217</v>
+        <v>211</v>
       </c>
       <c r="B102" t="s">
-        <v>218</v>
+        <v>212</v>
       </c>
       <c r="C102" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="D102" t="s">
-        <v>216</v>
+        <v>212</v>
       </c>
       <c r="E102" t="s">
         <v>109</v>
@@ -3433,111 +3436,117 @@
     </row>
     <row r="103" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A103" t="s">
-        <v>219</v>
+        <v>213</v>
       </c>
       <c r="B103" t="s">
-        <v>220</v>
+        <v>214</v>
       </c>
       <c r="C103" t="s">
-        <v>220</v>
+        <v>176</v>
       </c>
       <c r="D103" t="s">
-        <v>178</v>
+        <v>215</v>
+      </c>
+      <c r="E103" t="s">
+        <v>109</v>
       </c>
     </row>
     <row r="104" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A104" t="s">
-        <v>221</v>
+        <v>216</v>
       </c>
       <c r="B104" t="s">
-        <v>222</v>
+        <v>217</v>
       </c>
       <c r="C104" t="s">
-        <v>223</v>
+        <v>176</v>
       </c>
       <c r="D104" t="s">
-        <v>222</v>
+        <v>215</v>
+      </c>
+      <c r="E104" t="s">
+        <v>109</v>
       </c>
     </row>
     <row r="105" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A105" t="s">
-        <v>224</v>
+        <v>218</v>
       </c>
       <c r="B105" t="s">
-        <v>225</v>
+        <v>219</v>
       </c>
       <c r="C105" t="s">
-        <v>223</v>
+        <v>219</v>
       </c>
       <c r="D105" t="s">
-        <v>225</v>
+        <v>177</v>
       </c>
     </row>
     <row r="106" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A106" t="s">
-        <v>226</v>
+        <v>220</v>
       </c>
       <c r="B106" t="s">
-        <v>227</v>
+        <v>221</v>
       </c>
       <c r="C106" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="D106" t="s">
-        <v>227</v>
+        <v>221</v>
       </c>
     </row>
     <row r="107" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A107" t="s">
-        <v>228</v>
+        <v>223</v>
       </c>
       <c r="B107" t="s">
-        <v>229</v>
+        <v>224</v>
       </c>
       <c r="C107" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="D107" t="s">
-        <v>230</v>
+        <v>224</v>
       </c>
     </row>
     <row r="108" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A108" t="s">
-        <v>231</v>
+        <v>225</v>
       </c>
       <c r="B108" t="s">
-        <v>232</v>
+        <v>226</v>
       </c>
       <c r="C108" t="s">
-        <v>233</v>
+        <v>222</v>
       </c>
       <c r="D108" t="s">
-        <v>234</v>
+        <v>226</v>
       </c>
     </row>
     <row r="109" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A109" t="s">
-        <v>235</v>
+        <v>227</v>
       </c>
       <c r="B109" t="s">
-        <v>236</v>
+        <v>228</v>
       </c>
       <c r="C109" t="s">
-        <v>233</v>
+        <v>222</v>
       </c>
       <c r="D109" t="s">
-        <v>234</v>
+        <v>229</v>
       </c>
     </row>
     <row r="110" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A110" t="s">
-        <v>237</v>
+        <v>230</v>
       </c>
       <c r="B110" t="s">
-        <v>238</v>
+        <v>231</v>
       </c>
       <c r="C110" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="D110" t="s">
         <v>233</v>
@@ -3545,218 +3554,212 @@
     </row>
     <row r="111" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A111" t="s">
-        <v>239</v>
+        <v>234</v>
       </c>
       <c r="B111" t="s">
-        <v>240</v>
+        <v>235</v>
       </c>
       <c r="C111" t="s">
-        <v>241</v>
+        <v>232</v>
       </c>
       <c r="D111" t="s">
-        <v>242</v>
+        <v>233</v>
       </c>
     </row>
     <row r="112" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A112" t="s">
-        <v>243</v>
+        <v>236</v>
       </c>
       <c r="B112" t="s">
-        <v>244</v>
+        <v>237</v>
       </c>
       <c r="C112" t="s">
-        <v>241</v>
+        <v>232</v>
       </c>
       <c r="D112" t="s">
-        <v>242</v>
+        <v>232</v>
       </c>
     </row>
     <row r="113" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A113" t="s">
-        <v>245</v>
+        <v>238</v>
       </c>
       <c r="B113" t="s">
-        <v>246</v>
+        <v>239</v>
       </c>
       <c r="C113" t="s">
+        <v>240</v>
+      </c>
+      <c r="D113" t="s">
         <v>241</v>
-      </c>
-      <c r="D113" t="s">
-        <v>242</v>
       </c>
     </row>
     <row r="114" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A114" t="s">
-        <v>247</v>
+        <v>242</v>
       </c>
       <c r="B114" t="s">
-        <v>248</v>
+        <v>243</v>
       </c>
       <c r="C114" t="s">
+        <v>240</v>
+      </c>
+      <c r="D114" t="s">
         <v>241</v>
-      </c>
-      <c r="D114" t="s">
-        <v>242</v>
       </c>
     </row>
     <row r="115" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A115" t="s">
-        <v>249</v>
+        <v>244</v>
       </c>
       <c r="B115" t="s">
-        <v>250</v>
+        <v>245</v>
       </c>
       <c r="C115" t="s">
+        <v>240</v>
+      </c>
+      <c r="D115" t="s">
         <v>241</v>
-      </c>
-      <c r="D115" t="s">
-        <v>242</v>
       </c>
     </row>
     <row r="116" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A116" t="s">
-        <v>251</v>
+        <v>246</v>
       </c>
       <c r="B116" t="s">
-        <v>242</v>
+        <v>247</v>
       </c>
       <c r="C116" t="s">
+        <v>240</v>
+      </c>
+      <c r="D116" t="s">
         <v>241</v>
-      </c>
-      <c r="D116" t="s">
-        <v>242</v>
       </c>
     </row>
     <row r="117" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A117" t="s">
-        <v>252</v>
+        <v>248</v>
       </c>
       <c r="B117" t="s">
-        <v>253</v>
+        <v>249</v>
       </c>
       <c r="C117" t="s">
+        <v>240</v>
+      </c>
+      <c r="D117" t="s">
         <v>241</v>
-      </c>
-      <c r="D117" t="s">
-        <v>253</v>
       </c>
     </row>
     <row r="118" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A118" t="s">
-        <v>254</v>
+        <v>250</v>
       </c>
       <c r="B118" t="s">
-        <v>255</v>
+        <v>241</v>
       </c>
       <c r="C118" t="s">
+        <v>240</v>
+      </c>
+      <c r="D118" t="s">
         <v>241</v>
-      </c>
-      <c r="D118" t="s">
-        <v>230</v>
       </c>
     </row>
     <row r="119" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A119" t="s">
-        <v>256</v>
+        <v>251</v>
       </c>
       <c r="B119" t="s">
-        <v>257</v>
+        <v>252</v>
       </c>
       <c r="C119" t="s">
-        <v>258</v>
+        <v>240</v>
       </c>
       <c r="D119" t="s">
-        <v>259</v>
+        <v>252</v>
       </c>
     </row>
     <row r="120" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A120" t="s">
-        <v>260</v>
+        <v>253</v>
       </c>
       <c r="B120" t="s">
-        <v>261</v>
+        <v>254</v>
       </c>
       <c r="C120" t="s">
-        <v>258</v>
+        <v>240</v>
       </c>
       <c r="D120" t="s">
-        <v>261</v>
+        <v>229</v>
       </c>
     </row>
     <row r="121" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A121" t="s">
-        <v>262</v>
+        <v>255</v>
       </c>
       <c r="B121" t="s">
-        <v>263</v>
+        <v>256</v>
       </c>
       <c r="C121" t="s">
+        <v>257</v>
+      </c>
+      <c r="D121" t="s">
         <v>258</v>
-      </c>
-      <c r="D121" t="s">
-        <v>263</v>
       </c>
     </row>
     <row r="122" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A122" t="s">
-        <v>264</v>
+        <v>259</v>
       </c>
       <c r="B122" t="s">
-        <v>265</v>
+        <v>260</v>
       </c>
       <c r="C122" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="D122" t="s">
-        <v>230</v>
+        <v>260</v>
       </c>
     </row>
     <row r="123" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A123" t="s">
-        <v>266</v>
+        <v>261</v>
       </c>
       <c r="B123" t="s">
-        <v>267</v>
+        <v>262</v>
       </c>
       <c r="C123" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="D123" t="s">
-        <v>267</v>
-      </c>
-      <c r="E123" t="s">
-        <v>109</v>
+        <v>262</v>
       </c>
     </row>
     <row r="124" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A124" t="s">
-        <v>268</v>
+        <v>263</v>
       </c>
       <c r="B124" t="s">
-        <v>269</v>
+        <v>264</v>
       </c>
       <c r="C124" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="D124" t="s">
-        <v>269</v>
-      </c>
-      <c r="E124" t="s">
-        <v>109</v>
+        <v>229</v>
       </c>
     </row>
     <row r="125" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A125" t="s">
-        <v>270</v>
+        <v>265</v>
       </c>
       <c r="B125" t="s">
-        <v>271</v>
+        <v>266</v>
       </c>
       <c r="C125" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="D125" t="s">
-        <v>230</v>
+        <v>266</v>
       </c>
       <c r="E125" t="s">
         <v>109</v>
@@ -3764,16 +3767,16 @@
     </row>
     <row r="126" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A126" t="s">
-        <v>272</v>
+        <v>267</v>
       </c>
       <c r="B126" t="s">
-        <v>273</v>
+        <v>268</v>
       </c>
       <c r="C126" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="D126" t="s">
-        <v>274</v>
+        <v>268</v>
       </c>
       <c r="E126" t="s">
         <v>109</v>
@@ -3781,16 +3784,16 @@
     </row>
     <row r="127" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A127" t="s">
-        <v>275</v>
+        <v>269</v>
       </c>
       <c r="B127" t="s">
-        <v>276</v>
+        <v>270</v>
       </c>
       <c r="C127" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="D127" t="s">
-        <v>277</v>
+        <v>229</v>
       </c>
       <c r="E127" t="s">
         <v>109</v>
@@ -3798,878 +3801,912 @@
     </row>
     <row r="128" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A128" t="s">
-        <v>278</v>
+        <v>271</v>
       </c>
       <c r="B128" t="s">
-        <v>279</v>
+        <v>272</v>
       </c>
       <c r="C128" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="D128" t="s">
-        <v>277</v>
+        <v>273</v>
       </c>
       <c r="E128" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="129" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="129" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A129" t="s">
+        <v>274</v>
+      </c>
+      <c r="B129" t="s">
+        <v>275</v>
+      </c>
+      <c r="C129" t="s">
+        <v>257</v>
+      </c>
+      <c r="D129" t="s">
+        <v>276</v>
+      </c>
+      <c r="E129" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="130" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A130" t="s">
+        <v>277</v>
+      </c>
+      <c r="B130" t="s">
+        <v>278</v>
+      </c>
+      <c r="C130" t="s">
+        <v>257</v>
+      </c>
+      <c r="D130" t="s">
+        <v>276</v>
+      </c>
+      <c r="E130" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="131" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A131" t="s">
+        <v>279</v>
+      </c>
+      <c r="B131" t="s">
         <v>280</v>
       </c>
-      <c r="B129" t="s">
+      <c r="C131" t="s">
+        <v>257</v>
+      </c>
+      <c r="D131" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="132" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A132" t="s">
         <v>281</v>
       </c>
-      <c r="C129" t="s">
-        <v>258</v>
-      </c>
-      <c r="D129" t="s">
-        <v>274</v>
-      </c>
-    </row>
-    <row r="130" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A130" t="s">
+      <c r="B132" t="s">
         <v>282</v>
       </c>
-      <c r="B130" t="s">
+      <c r="C132" t="s">
+        <v>282</v>
+      </c>
+      <c r="D132" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="133" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A133" t="s">
         <v>283</v>
       </c>
-      <c r="C130" t="s">
-        <v>283</v>
-      </c>
-      <c r="D130" t="s">
-        <v>283</v>
-      </c>
-    </row>
-    <row r="131" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A131" t="s">
+      <c r="B133" t="s">
         <v>284</v>
       </c>
-      <c r="B131" t="s">
+      <c r="C133" t="s">
         <v>285</v>
       </c>
-      <c r="C131" t="s">
+      <c r="D133" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="134" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A134" t="s">
         <v>286</v>
       </c>
-      <c r="D131" t="s">
-        <v>286</v>
-      </c>
-    </row>
-    <row r="132" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A132" t="s">
+      <c r="B134" t="s">
         <v>287</v>
       </c>
-      <c r="B132" t="s">
+      <c r="C134" t="s">
+        <v>285</v>
+      </c>
+      <c r="D134" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="135" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A135" t="s">
         <v>288</v>
       </c>
-      <c r="C132" t="s">
-        <v>286</v>
-      </c>
-      <c r="D132" t="s">
-        <v>286</v>
-      </c>
-    </row>
-    <row r="133" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A133" t="s">
+      <c r="B135" t="s">
         <v>289</v>
       </c>
-      <c r="B133" t="s">
+      <c r="C135" t="s">
         <v>290</v>
       </c>
-      <c r="C133" t="s">
+      <c r="D135" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="136" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A136" t="s">
         <v>291</v>
       </c>
-      <c r="D133" t="s">
-        <v>291</v>
-      </c>
-    </row>
-    <row r="134" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A134" t="s">
+      <c r="B136" t="s">
         <v>292</v>
       </c>
-      <c r="B134" t="s">
+      <c r="C136" t="s">
+        <v>290</v>
+      </c>
+      <c r="D136" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="137" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A137" t="s">
         <v>293</v>
       </c>
-      <c r="C134" t="s">
-        <v>291</v>
-      </c>
-      <c r="D134" t="s">
-        <v>291</v>
-      </c>
-    </row>
-    <row r="135" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A135" t="s">
+      <c r="B137" t="s">
         <v>294</v>
       </c>
-      <c r="B135" t="s">
+      <c r="C137" t="s">
+        <v>290</v>
+      </c>
+      <c r="D137" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="138" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A138" t="s">
         <v>295</v>
       </c>
-      <c r="C135" t="s">
-        <v>291</v>
-      </c>
-      <c r="D135" t="s">
-        <v>291</v>
-      </c>
-    </row>
-    <row r="136" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A136" t="s">
+      <c r="B138" t="s">
         <v>296</v>
       </c>
-      <c r="B136" t="s">
+      <c r="C138" t="s">
+        <v>290</v>
+      </c>
+      <c r="D138" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="139" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A139" t="s">
         <v>297</v>
       </c>
-      <c r="C136" t="s">
-        <v>291</v>
-      </c>
-      <c r="D136" t="s">
-        <v>291</v>
-      </c>
-    </row>
-    <row r="137" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A137" t="s">
+      <c r="B139" t="s">
         <v>298</v>
       </c>
-      <c r="B137" t="s">
+      <c r="C139" t="s">
+        <v>290</v>
+      </c>
+      <c r="D139" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="140" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A140" t="s">
         <v>299</v>
       </c>
-      <c r="C137" t="s">
-        <v>291</v>
-      </c>
-      <c r="D137" t="s">
-        <v>291</v>
-      </c>
-    </row>
-    <row r="138" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A138" t="s">
+      <c r="B140" t="s">
         <v>300</v>
       </c>
-      <c r="B138" t="s">
+      <c r="C140" t="s">
+        <v>290</v>
+      </c>
+      <c r="D140" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="141" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A141" t="s">
         <v>301</v>
       </c>
-      <c r="C138" t="s">
-        <v>291</v>
-      </c>
-      <c r="D138" t="s">
-        <v>291</v>
-      </c>
-    </row>
-    <row r="139" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A139" t="s">
+      <c r="B141" t="s">
         <v>302</v>
       </c>
-      <c r="B139" t="s">
+      <c r="C141" t="s">
+        <v>298</v>
+      </c>
+      <c r="D141" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="142" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A142" t="s">
         <v>303</v>
       </c>
-      <c r="C139" t="s">
-        <v>299</v>
-      </c>
-      <c r="D139" t="s">
-        <v>299</v>
-      </c>
-    </row>
-    <row r="140" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A140" t="s">
+      <c r="B142" t="s">
         <v>304</v>
       </c>
-      <c r="B140" t="s">
+      <c r="C142" t="s">
         <v>305</v>
       </c>
-      <c r="C140" t="s">
+      <c r="D142" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="143" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A143" t="s">
         <v>306</v>
       </c>
-      <c r="D140" t="s">
-        <v>306</v>
-      </c>
-    </row>
-    <row r="141" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A141" t="s">
+      <c r="B143" t="s">
         <v>307</v>
       </c>
-      <c r="B141" t="s">
+      <c r="C143" t="s">
+        <v>305</v>
+      </c>
+      <c r="D143" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="144" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A144" t="s">
         <v>308</v>
       </c>
-      <c r="C141" t="s">
-        <v>306</v>
-      </c>
-      <c r="D141" t="s">
-        <v>306</v>
-      </c>
-    </row>
-    <row r="142" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A142" t="s">
+      <c r="B144" t="s">
         <v>309</v>
       </c>
-      <c r="B142" t="s">
-        <v>310</v>
-      </c>
-      <c r="C142" t="s">
-        <v>306</v>
-      </c>
-      <c r="D142" t="s">
-        <v>306</v>
-      </c>
-    </row>
-    <row r="143" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A143" t="s">
-        <v>311</v>
-      </c>
-      <c r="B143" t="s">
-        <v>312</v>
-      </c>
-      <c r="C143" t="s">
-        <v>306</v>
-      </c>
-      <c r="D143" t="s">
-        <v>306</v>
-      </c>
-    </row>
-    <row r="144" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A144" t="s">
-        <v>313</v>
-      </c>
-      <c r="B144" t="s">
-        <v>314</v>
-      </c>
       <c r="C144" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="D144" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="145" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A145" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
       <c r="B145" t="s">
-        <v>316</v>
+        <v>311</v>
       </c>
       <c r="C145" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="D145" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="146" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A146" t="s">
-        <v>317</v>
+        <v>312</v>
       </c>
       <c r="B146" t="s">
-        <v>318</v>
+        <v>313</v>
       </c>
       <c r="C146" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="D146" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="147" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A147" t="s">
-        <v>319</v>
+        <v>314</v>
       </c>
       <c r="B147" t="s">
-        <v>320</v>
+        <v>315</v>
       </c>
       <c r="C147" t="s">
-        <v>320</v>
+        <v>305</v>
       </c>
       <c r="D147" t="s">
-        <v>320</v>
+        <v>305</v>
       </c>
     </row>
     <row r="148" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A148" t="s">
-        <v>321</v>
+        <v>316</v>
       </c>
       <c r="B148" t="s">
-        <v>322</v>
+        <v>317</v>
       </c>
       <c r="C148" t="s">
-        <v>322</v>
+        <v>305</v>
       </c>
       <c r="D148" t="s">
-        <v>322</v>
+        <v>305</v>
       </c>
     </row>
     <row r="149" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A149" t="s">
-        <v>323</v>
+        <v>318</v>
       </c>
       <c r="B149" t="s">
-        <v>324</v>
+        <v>319</v>
       </c>
       <c r="C149" t="s">
-        <v>324</v>
+        <v>319</v>
       </c>
       <c r="D149" t="s">
-        <v>325</v>
+        <v>319</v>
       </c>
     </row>
     <row r="150" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A150" t="s">
-        <v>326</v>
+        <v>320</v>
       </c>
       <c r="B150" t="s">
-        <v>327</v>
+        <v>321</v>
       </c>
       <c r="C150" t="s">
-        <v>327</v>
+        <v>321</v>
       </c>
       <c r="D150" t="s">
-        <v>325</v>
+        <v>321</v>
       </c>
     </row>
     <row r="151" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A151" t="s">
-        <v>328</v>
+        <v>322</v>
       </c>
       <c r="B151" t="s">
-        <v>329</v>
+        <v>323</v>
       </c>
       <c r="C151" t="s">
-        <v>329</v>
+        <v>323</v>
       </c>
       <c r="D151" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
     </row>
     <row r="152" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A152" t="s">
-        <v>330</v>
+        <v>325</v>
       </c>
       <c r="B152" t="s">
-        <v>331</v>
+        <v>326</v>
       </c>
       <c r="C152" t="s">
-        <v>331</v>
+        <v>326</v>
       </c>
       <c r="D152" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
     </row>
     <row r="153" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A153" t="s">
-        <v>332</v>
+        <v>327</v>
       </c>
       <c r="B153" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="C153" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="D153" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
     </row>
     <row r="154" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A154" t="s">
-        <v>334</v>
+        <v>329</v>
       </c>
       <c r="B154" t="s">
-        <v>335</v>
+        <v>330</v>
       </c>
       <c r="C154" t="s">
-        <v>335</v>
+        <v>330</v>
       </c>
       <c r="D154" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
     </row>
     <row r="155" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A155" t="s">
-        <v>336</v>
+        <v>331</v>
       </c>
       <c r="B155" t="s">
-        <v>337</v>
+        <v>332</v>
       </c>
       <c r="C155" t="s">
-        <v>337</v>
+        <v>332</v>
       </c>
       <c r="D155" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
     </row>
     <row r="156" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A156" t="s">
-        <v>338</v>
+        <v>333</v>
       </c>
       <c r="B156" t="s">
-        <v>339</v>
+        <v>334</v>
       </c>
       <c r="C156" t="s">
-        <v>339</v>
+        <v>334</v>
       </c>
       <c r="D156" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
     </row>
     <row r="157" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A157" t="s">
-        <v>340</v>
+        <v>335</v>
       </c>
       <c r="B157" t="s">
-        <v>341</v>
+        <v>336</v>
       </c>
       <c r="C157" t="s">
-        <v>341</v>
+        <v>336</v>
       </c>
       <c r="D157" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
     </row>
     <row r="158" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A158" t="s">
-        <v>342</v>
+        <v>337</v>
       </c>
       <c r="B158" t="s">
-        <v>343</v>
+        <v>338</v>
       </c>
       <c r="C158" t="s">
-        <v>343</v>
+        <v>338</v>
       </c>
       <c r="D158" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
     </row>
     <row r="159" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A159" t="s">
-        <v>344</v>
+        <v>339</v>
       </c>
       <c r="B159" t="s">
-        <v>345</v>
+        <v>340</v>
       </c>
       <c r="C159" t="s">
-        <v>345</v>
+        <v>340</v>
       </c>
       <c r="D159" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
     </row>
     <row r="160" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A160" t="s">
-        <v>346</v>
+        <v>341</v>
       </c>
       <c r="B160" t="s">
-        <v>347</v>
+        <v>342</v>
       </c>
       <c r="C160" t="s">
-        <v>347</v>
+        <v>342</v>
       </c>
       <c r="D160" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
     </row>
     <row r="161" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A161" t="s">
-        <v>348</v>
+        <v>343</v>
       </c>
       <c r="B161" t="s">
-        <v>349</v>
+        <v>344</v>
       </c>
       <c r="C161" t="s">
-        <v>349</v>
+        <v>344</v>
       </c>
       <c r="D161" t="s">
-        <v>349</v>
+        <v>324</v>
       </c>
     </row>
     <row r="162" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A162" t="s">
-        <v>350</v>
+        <v>345</v>
       </c>
       <c r="B162" t="s">
-        <v>351</v>
+        <v>346</v>
       </c>
       <c r="C162" t="s">
-        <v>351</v>
+        <v>346</v>
       </c>
       <c r="D162" t="s">
-        <v>351</v>
+        <v>324</v>
       </c>
     </row>
     <row r="163" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A163" t="s">
-        <v>352</v>
+        <v>347</v>
       </c>
       <c r="B163" t="s">
-        <v>353</v>
+        <v>348</v>
       </c>
       <c r="C163" t="s">
-        <v>353</v>
+        <v>348</v>
       </c>
       <c r="D163" t="s">
-        <v>353</v>
+        <v>348</v>
       </c>
     </row>
     <row r="164" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A164" s="3" t="s">
-        <v>354</v>
-      </c>
-      <c r="B164" s="3" t="s">
-        <v>355</v>
-      </c>
-      <c r="C164" s="3" t="s">
-        <v>355</v>
+      <c r="A164" t="s">
+        <v>349</v>
+      </c>
+      <c r="B164" t="s">
+        <v>350</v>
+      </c>
+      <c r="C164" t="s">
+        <v>350</v>
       </c>
       <c r="D164" t="s">
-        <v>355</v>
+        <v>350</v>
       </c>
     </row>
     <row r="165" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A165" t="s">
-        <v>356</v>
+        <v>351</v>
       </c>
       <c r="B165" t="s">
-        <v>357</v>
+        <v>352</v>
       </c>
       <c r="C165" t="s">
-        <v>357</v>
+        <v>352</v>
       </c>
       <c r="D165" t="s">
-        <v>357</v>
+        <v>352</v>
       </c>
     </row>
     <row r="166" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A166" t="s">
-        <v>358</v>
-      </c>
-      <c r="B166" t="s">
-        <v>359</v>
-      </c>
-      <c r="C166" t="s">
-        <v>360</v>
+      <c r="A166" s="3" t="s">
+        <v>353</v>
+      </c>
+      <c r="B166" s="3" t="s">
+        <v>354</v>
+      </c>
+      <c r="C166" s="3" t="s">
+        <v>354</v>
       </c>
       <c r="D166" t="s">
-        <v>360</v>
+        <v>354</v>
       </c>
     </row>
     <row r="167" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A167" t="s">
-        <v>361</v>
+        <v>355</v>
       </c>
       <c r="B167" t="s">
-        <v>362</v>
+        <v>356</v>
       </c>
       <c r="C167" t="s">
-        <v>360</v>
+        <v>356</v>
       </c>
       <c r="D167" t="s">
-        <v>360</v>
+        <v>356</v>
       </c>
     </row>
     <row r="168" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A168" t="s">
-        <v>363</v>
+        <v>357</v>
       </c>
       <c r="B168" t="s">
-        <v>364</v>
+        <v>358</v>
       </c>
       <c r="C168" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="D168" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
     </row>
     <row r="169" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A169" t="s">
-        <v>365</v>
+        <v>360</v>
       </c>
       <c r="B169" t="s">
-        <v>366</v>
+        <v>361</v>
       </c>
       <c r="C169" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="D169" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
     </row>
     <row r="170" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A170" t="s">
-        <v>367</v>
+        <v>362</v>
       </c>
       <c r="B170" t="s">
-        <v>368</v>
+        <v>363</v>
       </c>
       <c r="C170" t="s">
-        <v>368</v>
+        <v>359</v>
       </c>
       <c r="D170" t="s">
-        <v>368</v>
+        <v>359</v>
       </c>
     </row>
     <row r="171" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A171" t="s">
-        <v>369</v>
+        <v>364</v>
       </c>
       <c r="B171" t="s">
-        <v>368</v>
+        <v>365</v>
       </c>
       <c r="C171" t="s">
-        <v>368</v>
+        <v>359</v>
       </c>
       <c r="D171" t="s">
-        <v>368</v>
+        <v>359</v>
       </c>
     </row>
     <row r="172" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A172" t="s">
-        <v>370</v>
+        <v>366</v>
       </c>
       <c r="B172" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="C172" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="D172" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
     </row>
     <row r="173" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A173" t="s">
-        <v>371</v>
+        <v>368</v>
       </c>
       <c r="B173" t="s">
-        <v>372</v>
+        <v>367</v>
       </c>
       <c r="C173" t="s">
-        <v>372</v>
+        <v>367</v>
       </c>
       <c r="D173" t="s">
-        <v>372</v>
+        <v>367</v>
       </c>
     </row>
     <row r="174" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A174" t="s">
-        <v>373</v>
+        <v>369</v>
       </c>
       <c r="B174" t="s">
-        <v>374</v>
+        <v>367</v>
       </c>
       <c r="C174" t="s">
-        <v>374</v>
+        <v>367</v>
       </c>
       <c r="D174" t="s">
-        <v>374</v>
+        <v>367</v>
       </c>
     </row>
     <row r="175" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A175" t="s">
-        <v>375</v>
+        <v>370</v>
       </c>
       <c r="B175" t="s">
-        <v>376</v>
+        <v>371</v>
       </c>
       <c r="C175" t="s">
-        <v>376</v>
+        <v>371</v>
       </c>
       <c r="D175" t="s">
-        <v>376</v>
+        <v>371</v>
       </c>
     </row>
     <row r="176" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A176" t="s">
-        <v>377</v>
+        <v>372</v>
       </c>
       <c r="B176" t="s">
-        <v>378</v>
+        <v>373</v>
       </c>
       <c r="C176" t="s">
-        <v>378</v>
+        <v>373</v>
       </c>
       <c r="D176" t="s">
-        <v>378</v>
+        <v>373</v>
       </c>
     </row>
     <row r="177" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A177" t="s">
-        <v>379</v>
+        <v>374</v>
       </c>
       <c r="B177" t="s">
-        <v>380</v>
+        <v>375</v>
       </c>
       <c r="C177" t="s">
-        <v>380</v>
+        <v>375</v>
       </c>
       <c r="D177" t="s">
-        <v>380</v>
+        <v>375</v>
       </c>
     </row>
     <row r="178" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A178" t="s">
-        <v>381</v>
+        <v>376</v>
       </c>
       <c r="B178" t="s">
-        <v>382</v>
+        <v>377</v>
       </c>
       <c r="C178" t="s">
-        <v>382</v>
+        <v>377</v>
       </c>
       <c r="D178" t="s">
-        <v>382</v>
+        <v>377</v>
       </c>
     </row>
     <row r="179" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A179" t="s">
-        <v>383</v>
+        <v>378</v>
       </c>
       <c r="B179" t="s">
-        <v>384</v>
+        <v>379</v>
       </c>
       <c r="C179" t="s">
-        <v>384</v>
+        <v>379</v>
       </c>
       <c r="D179" t="s">
-        <v>384</v>
+        <v>379</v>
       </c>
     </row>
     <row r="180" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A180" t="s">
-        <v>385</v>
+        <v>380</v>
       </c>
       <c r="B180" t="s">
-        <v>386</v>
+        <v>381</v>
       </c>
       <c r="C180" t="s">
-        <v>386</v>
+        <v>381</v>
       </c>
       <c r="D180" t="s">
-        <v>386</v>
+        <v>381</v>
       </c>
     </row>
     <row r="181" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A181" t="s">
-        <v>387</v>
+        <v>382</v>
       </c>
       <c r="B181" t="s">
-        <v>388</v>
+        <v>383</v>
       </c>
       <c r="C181" t="s">
-        <v>388</v>
+        <v>383</v>
       </c>
       <c r="D181" t="s">
-        <v>388</v>
+        <v>383</v>
       </c>
     </row>
     <row r="182" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A182" t="s">
-        <v>389</v>
+        <v>384</v>
       </c>
       <c r="B182" t="s">
-        <v>390</v>
+        <v>385</v>
       </c>
       <c r="C182" t="s">
-        <v>390</v>
+        <v>385</v>
       </c>
       <c r="D182" t="s">
-        <v>390</v>
+        <v>385</v>
       </c>
     </row>
     <row r="183" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A183" t="s">
-        <v>391</v>
+        <v>386</v>
       </c>
       <c r="B183" t="s">
-        <v>392</v>
+        <v>387</v>
       </c>
       <c r="C183" t="s">
-        <v>392</v>
+        <v>387</v>
       </c>
       <c r="D183" t="s">
-        <v>392</v>
+        <v>387</v>
       </c>
     </row>
     <row r="184" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A184" s="4" t="s">
-        <v>393</v>
-      </c>
-      <c r="B184" s="4" t="s">
-        <v>394</v>
-      </c>
-      <c r="C184" s="4" t="s">
-        <v>394</v>
-      </c>
-      <c r="D184" s="4" t="s">
-        <v>394</v>
-      </c>
-      <c r="E184" s="4"/>
+      <c r="A184" t="s">
+        <v>388</v>
+      </c>
+      <c r="B184" t="s">
+        <v>389</v>
+      </c>
+      <c r="C184" t="s">
+        <v>389</v>
+      </c>
+      <c r="D184" t="s">
+        <v>389</v>
+      </c>
     </row>
     <row r="185" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A185" t="s">
-        <v>395</v>
+        <v>390</v>
       </c>
       <c r="B185" t="s">
-        <v>396</v>
+        <v>391</v>
       </c>
       <c r="C185" t="s">
-        <v>291</v>
+        <v>391</v>
       </c>
       <c r="D185" t="s">
-        <v>291</v>
+        <v>391</v>
       </c>
     </row>
     <row r="186" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A186" t="s">
-        <v>397</v>
-      </c>
-      <c r="B186" t="s">
-        <v>398</v>
-      </c>
-      <c r="C186" t="s">
-        <v>291</v>
-      </c>
-      <c r="D186" t="s">
-        <v>291</v>
-      </c>
+      <c r="A186" s="4" t="s">
+        <v>392</v>
+      </c>
+      <c r="B186" s="4" t="s">
+        <v>393</v>
+      </c>
+      <c r="C186" s="4" t="s">
+        <v>393</v>
+      </c>
+      <c r="D186" s="4" t="s">
+        <v>393</v>
+      </c>
+      <c r="E186" s="4"/>
     </row>
     <row r="187" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A187" t="s">
-        <v>399</v>
+        <v>426</v>
       </c>
       <c r="B187" t="s">
-        <v>400</v>
+        <v>394</v>
       </c>
       <c r="C187" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="D187" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
     </row>
     <row r="188" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A188" t="s">
-        <v>401</v>
+        <v>427</v>
       </c>
       <c r="B188" t="s">
-        <v>402</v>
+        <v>395</v>
       </c>
       <c r="C188" t="s">
+        <v>290</v>
+      </c>
+      <c r="D188" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="189" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A189" t="s">
+        <v>396</v>
+      </c>
+      <c r="B189" t="s">
+        <v>397</v>
+      </c>
+      <c r="C189" t="s">
+        <v>290</v>
+      </c>
+      <c r="D189" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="190" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A190" t="s">
+        <v>398</v>
+      </c>
+      <c r="B190" t="s">
+        <v>399</v>
+      </c>
+      <c r="C190" t="s">
+        <v>176</v>
+      </c>
+      <c r="D190" t="s">
         <v>177</v>
       </c>
-      <c r="D188" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="189" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A189" t="s">
-        <v>428</v>
-      </c>
-      <c r="B189" t="s">
-        <v>173</v>
-      </c>
-      <c r="C189" t="s">
+    </row>
+    <row r="191" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A191" t="s">
+        <v>425</v>
+      </c>
+      <c r="B191" t="s">
         <v>172</v>
       </c>
-      <c r="D189" t="s">
-        <v>173</v>
+      <c r="C191" t="s">
+        <v>171</v>
+      </c>
+      <c r="D191" t="s">
+        <v>172</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E188" xr:uid="{00000000-0001-0000-0100-000000000000}"/>
+  <autoFilter ref="A1:E190" xr:uid="{00000000-0001-0000-0100-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>